<commit_message>
lazy frog tool commit
</commit_message>
<xml_diff>
--- a/credit_monthly_summary.xlsx
+++ b/credit_monthly_summary.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" tabRatio="600" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" tabRatio="600" firstSheet="3" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="CHASE #3444" sheetId="1" state="visible" r:id="rId1"/>
@@ -45,7 +45,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -60,19 +60,6 @@
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
@@ -140,18 +127,16 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="16" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -525,118 +510,118 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>CHASE #3444</t>
         </is>
       </c>
-      <c r="B1" s="7" t="n"/>
-      <c r="C1" s="7" t="n"/>
-      <c r="D1" s="7" t="n"/>
-      <c r="E1" s="7" t="n"/>
-      <c r="F1" s="7" t="n"/>
-      <c r="G1" s="7" t="n"/>
-      <c r="H1" s="7" t="n"/>
-      <c r="I1" s="7" t="n"/>
-      <c r="J1" s="7" t="n"/>
-      <c r="K1" s="7" t="n"/>
-      <c r="L1" s="7" t="n"/>
-      <c r="M1" s="7" t="n"/>
-      <c r="N1" s="7" t="n"/>
-      <c r="O1" s="7" t="n"/>
-      <c r="P1" s="7" t="n"/>
-      <c r="Q1" s="7" t="n"/>
-      <c r="R1" s="7" t="n"/>
-      <c r="S1" s="8" t="n"/>
+      <c r="B1" s="8" t="n"/>
+      <c r="C1" s="8" t="n"/>
+      <c r="D1" s="8" t="n"/>
+      <c r="E1" s="8" t="n"/>
+      <c r="F1" s="8" t="n"/>
+      <c r="G1" s="8" t="n"/>
+      <c r="H1" s="8" t="n"/>
+      <c r="I1" s="8" t="n"/>
+      <c r="J1" s="8" t="n"/>
+      <c r="K1" s="8" t="n"/>
+      <c r="L1" s="8" t="n"/>
+      <c r="M1" s="8" t="n"/>
+      <c r="N1" s="8" t="n"/>
+      <c r="O1" s="8" t="n"/>
+      <c r="P1" s="8" t="n"/>
+      <c r="Q1" s="8" t="n"/>
+      <c r="R1" s="8" t="n"/>
+      <c r="S1" s="9" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" s="6" t="n"/>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>BEGIN BALANCE</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>CASH / CHECK DEPOSIT</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>NO1 SUSHI 88 CORKBBO ACH</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>VEOLIA WATER</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>ORANGE &amp; ROCKLAND</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>WITHDRAWAL BRANCH 0964</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>AMAZON</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>BILL PAY:VEOLIA WATER NEW Y 200045 6BU1T6KR</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>BILL PAY:ORANGE &amp; ROCKLAND 136130 6BQ1P6KR</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>INTERNET TRF TO CLIENT-ADDED TRANSFER ACCOUNT</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="6" t="inlineStr">
         <is>
           <t>WITHDRAWAL BRANCH 0964 NEW YORK</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="6" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*NX6 SEATTLE WA</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*9O5 SEATTLE WA</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" s="6" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*SB8 SEATTLE WA</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="P2" s="6" t="inlineStr">
         <is>
           <t>NYS DTF PIT TAX PAYMNT</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="Q2" s="6" t="inlineStr">
         <is>
           <t>TOTAL CREDIT</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="R2" s="6" t="inlineStr">
         <is>
           <t>DEBIT</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="S2" s="6" t="inlineStr">
         <is>
           <t>ENDING BALANCE</t>
         </is>
@@ -1150,77 +1135,77 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Merchant</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>SEP</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>DEC</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>JAN</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>FEB</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>MAR</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>APR</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>MAY</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>JUN</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>JUL</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
@@ -1245,7 +1230,7 @@
       <c r="L2" s="3" t="n"/>
       <c r="M2" s="3" t="n"/>
       <c r="N2" s="3">
-        <f>SUM(B2:M2)</f>
+        <f>SUM(B2,C2,D2,E2,F2,G2,H2,I2,J2,K2,L2,M2)</f>
         <v/>
       </c>
       <c r="O2" s="1" t="inlineStr">
@@ -1273,7 +1258,7 @@
       <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="n"/>
       <c r="N3" s="3">
-        <f>SUM(B3:M3)</f>
+        <f>SUM(B3,C3,D3,E3,F3,G3,H3,I3,J3,K3,L3,M3)</f>
         <v/>
       </c>
       <c r="O3" s="1" t="inlineStr">
@@ -1301,7 +1286,7 @@
       <c r="L4" s="3" t="n"/>
       <c r="M4" s="3" t="n"/>
       <c r="N4" s="3">
-        <f>SUM(B4:M4)</f>
+        <f>SUM(B4,C4,D4,E4,F4,G4,H4,I4,J4,K4,L4,M4)</f>
         <v/>
       </c>
       <c r="O4" s="1" t="inlineStr">
@@ -1329,7 +1314,7 @@
       <c r="L5" s="3" t="n"/>
       <c r="M5" s="3" t="n"/>
       <c r="N5" s="3">
-        <f>SUM(B5:M5)</f>
+        <f>SUM(B5,C5,D5,E5,F5,G5,H5,I5,J5,K5,L5,M5)</f>
         <v/>
       </c>
       <c r="O5" s="1" t="inlineStr">
@@ -1357,7 +1342,7 @@
       <c r="L6" s="3" t="n"/>
       <c r="M6" s="3" t="n"/>
       <c r="N6" s="3">
-        <f>SUM(B6:M6)</f>
+        <f>SUM(B6,C6,D6,E6,F6,G6,H6,I6,J6,K6,L6,M6)</f>
         <v/>
       </c>
       <c r="O6" s="1" t="inlineStr">
@@ -1385,7 +1370,7 @@
       <c r="L7" s="3" t="n"/>
       <c r="M7" s="3" t="n"/>
       <c r="N7" s="3">
-        <f>SUM(B7:M7)</f>
+        <f>SUM(B7,C7,D7,E7,F7,G7,H7,I7,J7,K7,L7,M7)</f>
         <v/>
       </c>
       <c r="O7" s="1" t="inlineStr">
@@ -1413,7 +1398,7 @@
       <c r="L8" s="3" t="n"/>
       <c r="M8" s="3" t="n"/>
       <c r="N8" s="3">
-        <f>SUM(B8:M8)</f>
+        <f>SUM(B8,C8,D8,E8,F8,G8,H8,I8,J8,K8,L8,M8)</f>
         <v/>
       </c>
       <c r="O8" s="1" t="inlineStr">
@@ -1441,7 +1426,7 @@
       <c r="L9" s="3" t="n"/>
       <c r="M9" s="3" t="n"/>
       <c r="N9" s="3">
-        <f>SUM(B9:M9)</f>
+        <f>SUM(B9,C9,D9,E9,F9,G9,H9,I9,J9,K9,L9,M9)</f>
         <v/>
       </c>
       <c r="O9" s="1" t="inlineStr">
@@ -1469,7 +1454,7 @@
       <c r="L10" s="3" t="n"/>
       <c r="M10" s="3" t="n"/>
       <c r="N10" s="3">
-        <f>SUM(B10:M10)</f>
+        <f>SUM(B10,C10,D10,E10,F10,G10,H10,I10,J10,K10,L10,M10)</f>
         <v/>
       </c>
       <c r="O10" s="1" t="inlineStr">
@@ -1497,7 +1482,7 @@
       <c r="L11" s="3" t="n"/>
       <c r="M11" s="3" t="n"/>
       <c r="N11" s="3">
-        <f>SUM(B11:M11)</f>
+        <f>SUM(B11,C11,D11,E11,F11,G11,H11,I11,J11,K11,L11,M11)</f>
         <v/>
       </c>
       <c r="O11" s="1" t="inlineStr">
@@ -1525,7 +1510,7 @@
       <c r="L12" s="3" t="n"/>
       <c r="M12" s="3" t="n"/>
       <c r="N12" s="3">
-        <f>SUM(B12:M12)</f>
+        <f>SUM(B12,C12,D12,E12,F12,G12,H12,I12,J12,K12,L12,M12)</f>
         <v/>
       </c>
       <c r="O12" s="1" t="inlineStr">
@@ -1553,7 +1538,7 @@
       <c r="L13" s="3" t="n"/>
       <c r="M13" s="3" t="n"/>
       <c r="N13" s="3">
-        <f>SUM(B13:M13)</f>
+        <f>SUM(B13,C13,D13,E13,F13,G13,H13,I13,J13,K13,L13,M13)</f>
         <v/>
       </c>
       <c r="O13" s="1" t="inlineStr">
@@ -1581,7 +1566,7 @@
       <c r="L14" s="3" t="n"/>
       <c r="M14" s="3" t="n"/>
       <c r="N14" s="3">
-        <f>SUM(B14:M14)</f>
+        <f>SUM(B14,C14,D14,E14,F14,G14,H14,I14,J14,K14,L14,M14)</f>
         <v/>
       </c>
       <c r="O14" s="1" t="inlineStr">
@@ -1609,7 +1594,7 @@
       <c r="L15" s="3" t="n"/>
       <c r="M15" s="3" t="n"/>
       <c r="N15" s="3">
-        <f>SUM(B15:M15)</f>
+        <f>SUM(B15,C15,D15,E15,F15,G15,H15,I15,J15,K15,L15,M15)</f>
         <v/>
       </c>
       <c r="O15" s="1" t="inlineStr">
@@ -1637,7 +1622,7 @@
       <c r="L16" s="3" t="n"/>
       <c r="M16" s="3" t="n"/>
       <c r="N16" s="3">
-        <f>SUM(B16:M16)</f>
+        <f>SUM(B16,C16,D16,E16,F16,G16,H16,I16,J16,K16,L16,M16)</f>
         <v/>
       </c>
       <c r="O16" s="1" t="inlineStr">
@@ -1665,7 +1650,7 @@
       <c r="L17" s="3" t="n"/>
       <c r="M17" s="3" t="n"/>
       <c r="N17" s="3">
-        <f>SUM(B17:M17)</f>
+        <f>SUM(B17,C17,D17,E17,F17,G17,H17,I17,J17,K17,L17,M17)</f>
         <v/>
       </c>
       <c r="O17" s="1" t="inlineStr">
@@ -1693,7 +1678,7 @@
       <c r="L18" s="3" t="n"/>
       <c r="M18" s="3" t="n"/>
       <c r="N18" s="3">
-        <f>SUM(B18:M18)</f>
+        <f>SUM(B18,C18,D18,E18,F18,G18,H18,I18,J18,K18,L18,M18)</f>
         <v/>
       </c>
       <c r="O18" s="1" t="inlineStr">
@@ -1721,7 +1706,7 @@
       <c r="L19" s="3" t="n"/>
       <c r="M19" s="3" t="n"/>
       <c r="N19" s="3">
-        <f>SUM(B19:M19)</f>
+        <f>SUM(B19,C19,D19,E19,F19,G19,H19,I19,J19,K19,L19,M19)</f>
         <v/>
       </c>
       <c r="O19" s="1" t="inlineStr">
@@ -1749,7 +1734,7 @@
       <c r="L20" s="3" t="n"/>
       <c r="M20" s="3" t="n"/>
       <c r="N20" s="3">
-        <f>SUM(B20:M20)</f>
+        <f>SUM(B20,C20,D20,E20,F20,G20,H20,I20,J20,K20,L20,M20)</f>
         <v/>
       </c>
       <c r="O20" s="1" t="inlineStr">
@@ -1777,7 +1762,7 @@
       <c r="L21" s="3" t="n"/>
       <c r="M21" s="3" t="n"/>
       <c r="N21" s="3">
-        <f>SUM(B21:M21)</f>
+        <f>SUM(B21,C21,D21,E21,F21,G21,H21,I21,J21,K21,L21,M21)</f>
         <v/>
       </c>
       <c r="O21" s="1" t="inlineStr">
@@ -1805,7 +1790,7 @@
       <c r="L22" s="3" t="n"/>
       <c r="M22" s="3" t="n"/>
       <c r="N22" s="3">
-        <f>SUM(B22:M22)</f>
+        <f>SUM(B22,C22,D22,E22,F22,G22,H22,I22,J22,K22,L22,M22)</f>
         <v/>
       </c>
       <c r="O22" s="1" t="inlineStr">
@@ -1833,7 +1818,7 @@
       <c r="L23" s="3" t="n"/>
       <c r="M23" s="3" t="n"/>
       <c r="N23" s="3">
-        <f>SUM(B23:M23)</f>
+        <f>SUM(B23,C23,D23,E23,F23,G23,H23,I23,J23,K23,L23,M23)</f>
         <v/>
       </c>
       <c r="O23" s="1" t="inlineStr">
@@ -1861,7 +1846,7 @@
       <c r="L24" s="3" t="n"/>
       <c r="M24" s="3" t="n"/>
       <c r="N24" s="3">
-        <f>SUM(B24:M24)</f>
+        <f>SUM(B24,C24,D24,E24,F24,G24,H24,I24,J24,K24,L24,M24)</f>
         <v/>
       </c>
       <c r="O24" s="1" t="inlineStr">
@@ -1889,7 +1874,7 @@
       <c r="L25" s="3" t="n"/>
       <c r="M25" s="3" t="n"/>
       <c r="N25" s="3">
-        <f>SUM(B25:M25)</f>
+        <f>SUM(B25,C25,D25,E25,F25,G25,H25,I25,J25,K25,L25,M25)</f>
         <v/>
       </c>
       <c r="O25" s="1" t="inlineStr">
@@ -1917,7 +1902,7 @@
       <c r="L26" s="3" t="n"/>
       <c r="M26" s="3" t="n"/>
       <c r="N26" s="3">
-        <f>SUM(B26:M26)</f>
+        <f>SUM(B26,C26,D26,E26,F26,G26,H26,I26,J26,K26,L26,M26)</f>
         <v/>
       </c>
       <c r="O26" s="1" t="inlineStr">
@@ -1945,7 +1930,7 @@
       <c r="L27" s="3" t="n"/>
       <c r="M27" s="3" t="n"/>
       <c r="N27" s="3">
-        <f>SUM(B27:M27)</f>
+        <f>SUM(B27,C27,D27,E27,F27,G27,H27,I27,J27,K27,L27,M27)</f>
         <v/>
       </c>
       <c r="O27" s="1" t="inlineStr">
@@ -1973,7 +1958,7 @@
       <c r="L28" s="3" t="n"/>
       <c r="M28" s="3" t="n"/>
       <c r="N28" s="3">
-        <f>SUM(B28:M28)</f>
+        <f>SUM(B28,C28,D28,E28,F28,G28,H28,I28,J28,K28,L28,M28)</f>
         <v/>
       </c>
       <c r="O28" s="1" t="inlineStr">
@@ -2001,7 +1986,7 @@
       <c r="L29" s="3" t="n"/>
       <c r="M29" s="3" t="n"/>
       <c r="N29" s="3">
-        <f>SUM(B29:M29)</f>
+        <f>SUM(B29,C29,D29,E29,F29,G29,H29,I29,J29,K29,L29,M29)</f>
         <v/>
       </c>
       <c r="O29" s="1" t="inlineStr">
@@ -2029,7 +2014,7 @@
       <c r="L30" s="3" t="n"/>
       <c r="M30" s="3" t="n"/>
       <c r="N30" s="3">
-        <f>SUM(B30:M30)</f>
+        <f>SUM(B30,C30,D30,E30,F30,G30,H30,I30,J30,K30,L30,M30)</f>
         <v/>
       </c>
       <c r="O30" s="1" t="inlineStr">
@@ -2057,7 +2042,7 @@
       <c r="L31" s="3" t="n"/>
       <c r="M31" s="3" t="n"/>
       <c r="N31" s="3">
-        <f>SUM(B31:M31)</f>
+        <f>SUM(B31,C31,D31,E31,F31,G31,H31,I31,J31,K31,L31,M31)</f>
         <v/>
       </c>
       <c r="O31" s="1" t="inlineStr">
@@ -2085,7 +2070,7 @@
       <c r="L32" s="3" t="n"/>
       <c r="M32" s="3" t="n"/>
       <c r="N32" s="3">
-        <f>SUM(B32:M32)</f>
+        <f>SUM(B32,C32,D32,E32,F32,G32,H32,I32,J32,K32,L32,M32)</f>
         <v/>
       </c>
       <c r="O32" s="1" t="inlineStr">
@@ -2113,7 +2098,7 @@
       <c r="L33" s="3" t="n"/>
       <c r="M33" s="3" t="n"/>
       <c r="N33" s="3">
-        <f>SUM(B33:M33)</f>
+        <f>SUM(B33,C33,D33,E33,F33,G33,H33,I33,J33,K33,L33,M33)</f>
         <v/>
       </c>
       <c r="O33" s="1" t="inlineStr">
@@ -2141,7 +2126,7 @@
       <c r="L34" s="3" t="n"/>
       <c r="M34" s="3" t="n"/>
       <c r="N34" s="3">
-        <f>SUM(B34:M34)</f>
+        <f>SUM(B34,C34,D34,E34,F34,G34,H34,I34,J34,K34,L34,M34)</f>
         <v/>
       </c>
       <c r="O34" s="1" t="inlineStr">
@@ -2169,7 +2154,7 @@
       <c r="L35" s="3" t="n"/>
       <c r="M35" s="3" t="n"/>
       <c r="N35" s="3">
-        <f>SUM(B35:M35)</f>
+        <f>SUM(B35,C35,D35,E35,F35,G35,H35,I35,J35,K35,L35,M35)</f>
         <v/>
       </c>
       <c r="O35" s="1" t="inlineStr">
@@ -2197,7 +2182,7 @@
       <c r="L36" s="3" t="n"/>
       <c r="M36" s="3" t="n"/>
       <c r="N36" s="3">
-        <f>SUM(B36:M36)</f>
+        <f>SUM(B36,C36,D36,E36,F36,G36,H36,I36,J36,K36,L36,M36)</f>
         <v/>
       </c>
       <c r="O36" s="1" t="inlineStr">
@@ -2225,7 +2210,7 @@
       <c r="L37" s="3" t="n"/>
       <c r="M37" s="3" t="n"/>
       <c r="N37" s="3">
-        <f>SUM(B37:M37)</f>
+        <f>SUM(B37,C37,D37,E37,F37,G37,H37,I37,J37,K37,L37,M37)</f>
         <v/>
       </c>
       <c r="O37" s="1" t="inlineStr">
@@ -2253,7 +2238,7 @@
       <c r="L38" s="3" t="n"/>
       <c r="M38" s="3" t="n"/>
       <c r="N38" s="3">
-        <f>SUM(B38:M38)</f>
+        <f>SUM(B38,C38,D38,E38,F38,G38,H38,I38,J38,K38,L38,M38)</f>
         <v/>
       </c>
       <c r="O38" s="1" t="inlineStr">
@@ -2281,7 +2266,7 @@
       <c r="L39" s="3" t="n"/>
       <c r="M39" s="3" t="n"/>
       <c r="N39" s="3">
-        <f>SUM(B39:M39)</f>
+        <f>SUM(B39,C39,D39,E39,F39,G39,H39,I39,J39,K39,L39,M39)</f>
         <v/>
       </c>
       <c r="O39" s="1" t="inlineStr">
@@ -2309,7 +2294,7 @@
       <c r="L40" s="3" t="n"/>
       <c r="M40" s="3" t="n"/>
       <c r="N40" s="3">
-        <f>SUM(B40:M40)</f>
+        <f>SUM(B40,C40,D40,E40,F40,G40,H40,I40,J40,K40,L40,M40)</f>
         <v/>
       </c>
       <c r="O40" s="1" t="inlineStr">
@@ -2337,7 +2322,7 @@
       <c r="L41" s="3" t="n"/>
       <c r="M41" s="3" t="n"/>
       <c r="N41" s="3">
-        <f>SUM(B41:M41)</f>
+        <f>SUM(B41,C41,D41,E41,F41,G41,H41,I41,J41,K41,L41,M41)</f>
         <v/>
       </c>
       <c r="O41" s="1" t="n"/>
@@ -2348,56 +2333,56 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B42" s="9">
+      <c r="B42" s="5">
         <f>SUM(B2:B41)</f>
         <v/>
       </c>
-      <c r="C42" s="9">
+      <c r="C42" s="5">
         <f>SUM(C2:C41)</f>
         <v/>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="5">
         <f>SUM(D2:D41)</f>
         <v/>
       </c>
-      <c r="E42" s="9">
+      <c r="E42" s="5">
         <f>SUM(E2:E41)</f>
         <v/>
       </c>
-      <c r="F42" s="9">
+      <c r="F42" s="5">
         <f>SUM(F2:F41)</f>
         <v/>
       </c>
-      <c r="G42" s="9">
+      <c r="G42" s="5">
         <f>SUM(G2:G41)</f>
         <v/>
       </c>
-      <c r="H42" s="9">
+      <c r="H42" s="5">
         <f>SUM(H2:H41)</f>
         <v/>
       </c>
-      <c r="I42" s="9">
+      <c r="I42" s="5">
         <f>SUM(I2:I41)</f>
         <v/>
       </c>
-      <c r="J42" s="9">
+      <c r="J42" s="5">
         <f>SUM(J2:J41)</f>
         <v/>
       </c>
-      <c r="K42" s="9">
+      <c r="K42" s="5">
         <f>SUM(K2:K41)</f>
         <v/>
       </c>
-      <c r="L42" s="9">
+      <c r="L42" s="5">
         <f>SUM(L2:L41)</f>
         <v/>
       </c>
-      <c r="M42" s="9">
+      <c r="M42" s="5">
         <f>SUM(M2:M41)</f>
         <v/>
       </c>
-      <c r="N42" s="9">
-        <f>SUM(B42:M42)</f>
+      <c r="N42" s="5">
+        <f>SUM(B42,C42,D42,E42,F42,G42,H42,I42,J42,K42,L42,M42)</f>
         <v/>
       </c>
     </row>
@@ -2413,7 +2398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2432,14 +2417,14 @@
     <col width="40.7109375" bestFit="1" customWidth="1" min="14" max="14"/>
     <col width="40.42578125" bestFit="1" customWidth="1" min="15" max="15"/>
     <col width="24.7109375" bestFit="1" customWidth="1" min="16" max="16"/>
-    <col width="24.7109375" bestFit="1" customWidth="1" min="17" max="17"/>
-    <col width="24.7109375" bestFit="1" customWidth="1" min="18" max="18"/>
-    <col width="24.7109375" bestFit="1" customWidth="1" min="19" max="19"/>
+    <col width="13.85546875" bestFit="1" customWidth="1" min="17" max="17"/>
+    <col width="8.140625" bestFit="1" customWidth="1" min="18" max="18"/>
+    <col width="17.42578125" bestFit="1" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="n"/>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>CHASE #3444</t>
         </is>
@@ -2461,113 +2446,95 @@
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" s="6" t="n"/>
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>BEGIN BALANCE</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>CASH / CHECK DEPOSIT</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>NO1 SUSHI 88 CORKBBO ACH</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>VEOLIA WATER</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>ORANGE &amp; ROCKLAND</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>WITHDRAWAL BRANCH 0964</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>AMAZON</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>BILL PAY:VEOLIA WATER NEW Y 200045 6BU1T6KR</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>BILL PAY:ORANGE &amp; ROCKLAND 136130 6BQ1P6KR</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>INTERNET TRF TO CLIENT-ADDED TRANSFER ACCOUNT</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="6" t="inlineStr">
         <is>
           <t>WITHDRAWAL BRANCH 0964 NEW YORK</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M2" s="6" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*NX6 SEATTLE WA</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*9O5 SEATTLE WA</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" s="6" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*SB8 SEATTLE WA</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="P2" s="6" t="inlineStr">
         <is>
           <t>NYS DTF PIT TAX PAYMNT</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>KINDERCARE PORTLAND OR</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>AMAZON PRIME*ZH8618UZ3 AMZN.COM/BILL WA</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>IRS USATAXPYMT</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="Q2" s="6" t="inlineStr">
         <is>
           <t>TOTAL CREDIT</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr">
+      <c r="R2" s="6" t="inlineStr">
         <is>
           <t>DEBIT</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="S2" s="6" t="inlineStr">
         <is>
           <t>ENDING BALANCE</t>
         </is>
@@ -2596,16 +2563,13 @@
       <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="n"/>
       <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3" t="n"/>
+      <c r="Q3" s="3">
+        <f>SUM(C3:P3)</f>
+        <v/>
+      </c>
       <c r="R3" s="3" t="n"/>
-      <c r="S3" s="3" t="n"/>
-      <c r="T3" s="3">
-        <f>SUM(C3:S3)</f>
-        <v/>
-      </c>
-      <c r="U3" s="3" t="n"/>
-      <c r="V3" s="3">
-        <f>B3+T3-U3</f>
+      <c r="S3" s="3">
+        <f>B3+Q3-R3</f>
         <v/>
       </c>
     </row>
@@ -2633,16 +2597,13 @@
       <c r="N4" s="3" t="n"/>
       <c r="O4" s="3" t="n"/>
       <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3" t="n"/>
+      <c r="Q4" s="3">
+        <f>SUM(C4:P4)</f>
+        <v/>
+      </c>
       <c r="R4" s="3" t="n"/>
-      <c r="S4" s="3" t="n"/>
-      <c r="T4" s="3">
-        <f>SUM(C4:S4)</f>
-        <v/>
-      </c>
-      <c r="U4" s="3" t="n"/>
-      <c r="V4" s="3">
-        <f>B4+T4-U4</f>
+      <c r="S4" s="3">
+        <f>B4+Q4-R4</f>
         <v/>
       </c>
     </row>
@@ -2670,16 +2631,13 @@
       <c r="N5" s="3" t="n"/>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="n"/>
-      <c r="Q5" s="3" t="n"/>
+      <c r="Q5" s="3">
+        <f>SUM(C5:P5)</f>
+        <v/>
+      </c>
       <c r="R5" s="3" t="n"/>
-      <c r="S5" s="3" t="n"/>
-      <c r="T5" s="3">
-        <f>SUM(C5:S5)</f>
-        <v/>
-      </c>
-      <c r="U5" s="3" t="n"/>
-      <c r="V5" s="3">
-        <f>B5+T5-U5</f>
+      <c r="S5" s="3">
+        <f>B5+Q5-R5</f>
         <v/>
       </c>
     </row>
@@ -2694,65 +2652,26 @@
         <v/>
       </c>
       <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3">
-        <f>4000.00</f>
-        <v/>
-      </c>
+      <c r="D6" s="3" t="n"/>
       <c r="E6" s="3" t="n"/>
       <c r="F6" s="3" t="n"/>
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3">
-        <f>300.00</f>
-        <v/>
-      </c>
-      <c r="J6" s="3">
-        <f>350.00</f>
-        <v/>
-      </c>
-      <c r="K6" s="3">
-        <f>385.77+740.00</f>
-        <v/>
-      </c>
-      <c r="L6" s="3">
-        <f>1000.00+3200.00</f>
-        <v/>
-      </c>
-      <c r="M6" s="3">
-        <f>75.40</f>
-        <v/>
-      </c>
-      <c r="N6" s="3">
-        <f>26.57</f>
-        <v/>
-      </c>
-      <c r="O6" s="3">
-        <f>18.75</f>
-        <v/>
-      </c>
-      <c r="P6" s="3">
-        <f>200.00+200.00</f>
-        <v/>
-      </c>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="3" t="n"/>
+      <c r="N6" s="3" t="n"/>
+      <c r="O6" s="3" t="n"/>
+      <c r="P6" s="3" t="n"/>
       <c r="Q6" s="3">
-        <f>490.00</f>
-        <v/>
-      </c>
-      <c r="R6" s="3">
-        <f>16.25</f>
-        <v/>
-      </c>
+        <f>SUM(C6:P6)</f>
+        <v/>
+      </c>
+      <c r="R6" s="3" t="n"/>
       <c r="S6" s="3">
-        <f>800.00+800.00</f>
-        <v/>
-      </c>
-      <c r="T6" s="3">
-        <f>SUM(C6:S6)</f>
-        <v/>
-      </c>
-      <c r="U6" s="3" t="n"/>
-      <c r="V6" s="3">
-        <f>B6+T6-U6</f>
+        <f>B6+Q6-R6</f>
         <v/>
       </c>
     </row>
@@ -2780,16 +2699,13 @@
       <c r="N7" s="3" t="n"/>
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="n"/>
-      <c r="Q7" s="3" t="n"/>
+      <c r="Q7" s="3">
+        <f>SUM(C7:P7)</f>
+        <v/>
+      </c>
       <c r="R7" s="3" t="n"/>
-      <c r="S7" s="3" t="n"/>
-      <c r="T7" s="3">
-        <f>SUM(C7:S7)</f>
-        <v/>
-      </c>
-      <c r="U7" s="3" t="n"/>
-      <c r="V7" s="3">
-        <f>B7+T7-U7</f>
+      <c r="S7" s="3">
+        <f>B7+Q7-R7</f>
         <v/>
       </c>
     </row>
@@ -2817,16 +2733,13 @@
       <c r="N8" s="3" t="n"/>
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="n"/>
-      <c r="Q8" s="3" t="n"/>
+      <c r="Q8" s="3">
+        <f>SUM(C8:P8)</f>
+        <v/>
+      </c>
       <c r="R8" s="3" t="n"/>
-      <c r="S8" s="3" t="n"/>
-      <c r="T8" s="3">
-        <f>SUM(C8:S8)</f>
-        <v/>
-      </c>
-      <c r="U8" s="3" t="n"/>
-      <c r="V8" s="3">
-        <f>B8+T8-U8</f>
+      <c r="S8" s="3">
+        <f>B8+Q8-R8</f>
         <v/>
       </c>
     </row>
@@ -2854,16 +2767,13 @@
       <c r="N9" s="3" t="n"/>
       <c r="O9" s="3" t="n"/>
       <c r="P9" s="3" t="n"/>
-      <c r="Q9" s="3" t="n"/>
+      <c r="Q9" s="3">
+        <f>SUM(C9:P9)</f>
+        <v/>
+      </c>
       <c r="R9" s="3" t="n"/>
-      <c r="S9" s="3" t="n"/>
-      <c r="T9" s="3">
-        <f>SUM(C9:S9)</f>
-        <v/>
-      </c>
-      <c r="U9" s="3" t="n"/>
-      <c r="V9" s="3">
-        <f>B9+T9-U9</f>
+      <c r="S9" s="3">
+        <f>B9+Q9-R9</f>
         <v/>
       </c>
     </row>
@@ -2891,16 +2801,13 @@
       <c r="N10" s="3" t="n"/>
       <c r="O10" s="3" t="n"/>
       <c r="P10" s="3" t="n"/>
-      <c r="Q10" s="3" t="n"/>
+      <c r="Q10" s="3">
+        <f>SUM(C10:P10)</f>
+        <v/>
+      </c>
       <c r="R10" s="3" t="n"/>
-      <c r="S10" s="3" t="n"/>
-      <c r="T10" s="3">
-        <f>SUM(C10:S10)</f>
-        <v/>
-      </c>
-      <c r="U10" s="3" t="n"/>
-      <c r="V10" s="3">
-        <f>B10+T10-U10</f>
+      <c r="S10" s="3">
+        <f>B10+Q10-R10</f>
         <v/>
       </c>
     </row>
@@ -2928,16 +2835,13 @@
       <c r="N11" s="3" t="n"/>
       <c r="O11" s="3" t="n"/>
       <c r="P11" s="3" t="n"/>
-      <c r="Q11" s="3" t="n"/>
+      <c r="Q11" s="3">
+        <f>SUM(C11:P11)</f>
+        <v/>
+      </c>
       <c r="R11" s="3" t="n"/>
-      <c r="S11" s="3" t="n"/>
-      <c r="T11" s="3">
-        <f>SUM(C11:S11)</f>
-        <v/>
-      </c>
-      <c r="U11" s="3" t="n"/>
-      <c r="V11" s="3">
-        <f>B11+T11-U11</f>
+      <c r="S11" s="3">
+        <f>B11+Q11-R11</f>
         <v/>
       </c>
     </row>
@@ -2965,16 +2869,13 @@
       <c r="N12" s="3" t="n"/>
       <c r="O12" s="3" t="n"/>
       <c r="P12" s="3" t="n"/>
-      <c r="Q12" s="3" t="n"/>
+      <c r="Q12" s="3">
+        <f>SUM(C12:P12)</f>
+        <v/>
+      </c>
       <c r="R12" s="3" t="n"/>
-      <c r="S12" s="3" t="n"/>
-      <c r="T12" s="3">
-        <f>SUM(C12:S12)</f>
-        <v/>
-      </c>
-      <c r="U12" s="3" t="n"/>
-      <c r="V12" s="3">
-        <f>B12+T12-U12</f>
+      <c r="S12" s="3">
+        <f>B12+Q12-R12</f>
         <v/>
       </c>
     </row>
@@ -3002,16 +2903,13 @@
       <c r="N13" s="3" t="n"/>
       <c r="O13" s="3" t="n"/>
       <c r="P13" s="3" t="n"/>
-      <c r="Q13" s="3" t="n"/>
+      <c r="Q13" s="3">
+        <f>SUM(C13:P13)</f>
+        <v/>
+      </c>
       <c r="R13" s="3" t="n"/>
-      <c r="S13" s="3" t="n"/>
-      <c r="T13" s="3">
-        <f>SUM(C13:S13)</f>
-        <v/>
-      </c>
-      <c r="U13" s="3" t="n"/>
-      <c r="V13" s="3">
-        <f>B13+T13-U13</f>
+      <c r="S13" s="3">
+        <f>B13+Q13-R13</f>
         <v/>
       </c>
     </row>
@@ -3039,16 +2937,13 @@
       <c r="N14" s="3" t="n"/>
       <c r="O14" s="3" t="n"/>
       <c r="P14" s="3" t="n"/>
-      <c r="Q14" s="3" t="n"/>
+      <c r="Q14" s="3">
+        <f>SUM(C14:P14)</f>
+        <v/>
+      </c>
       <c r="R14" s="3" t="n"/>
-      <c r="S14" s="3" t="n"/>
-      <c r="T14" s="3">
-        <f>SUM(C14:S14)</f>
-        <v/>
-      </c>
-      <c r="U14" s="3" t="n"/>
-      <c r="V14" s="3">
-        <f>B14+T14-U14</f>
+      <c r="S14" s="3">
+        <f>B14+Q14-R14</f>
         <v/>
       </c>
     </row>
@@ -3124,19 +3019,7 @@
         <v/>
       </c>
       <c r="S15" s="3">
-        <f>SUM(S3:S14)</f>
-        <v/>
-      </c>
-      <c r="T15" s="3">
-        <f>SUM(T3:T14)</f>
-        <v/>
-      </c>
-      <c r="U15" s="3">
-        <f>SUM(U3:U14)</f>
-        <v/>
-      </c>
-      <c r="V15" s="3">
-        <f>V14</f>
+        <f>S14</f>
         <v/>
       </c>
     </row>
@@ -3151,7 +3034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3164,85 +3047,92 @@
     <col width="5" bestFit="1" customWidth="1" min="10" max="10"/>
     <col width="5.42578125" bestFit="1" customWidth="1" min="11" max="11"/>
     <col width="5" bestFit="1" customWidth="1" min="12" max="13"/>
-    <col width="8.140625" bestFit="1" customWidth="1" min="14" max="14"/>
-    <col width="15.5703125" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="6.28515625" bestFit="1" customWidth="1" min="14" max="14"/>
+    <col width="8.140625" bestFit="1" customWidth="1" min="15" max="15"/>
+    <col width="15.5703125" bestFit="1" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Merchant</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>SEP</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>DEC</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>JAN</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>FEB</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>MAR</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>APR</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>MAY</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>JUN</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>JUL</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="4" t="n">
+        <v>46234</v>
+      </c>
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
+      </c>
+      <c r="Q1" s="7" t="n">
+        <v>46240</v>
       </c>
     </row>
     <row r="2">
@@ -3263,11 +3153,12 @@
       <c r="K2" s="3" t="n"/>
       <c r="L2" s="3" t="n"/>
       <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3">
-        <f>SUM(B2:M2)</f>
-        <v/>
-      </c>
-      <c r="O2" s="1" t="inlineStr">
+      <c r="N2" s="3" t="n"/>
+      <c r="O2" s="3">
+        <f>SUM(B2,C2,D2,E2,F2,G2,H2,I2,J2,K2,L2,M2,N2,Q2)</f>
+        <v/>
+      </c>
+      <c r="P2" s="1" t="inlineStr">
         <is>
           <t>GERCORY</t>
         </is>
@@ -3285,23 +3176,31 @@
       <c r="E3" s="3" t="n"/>
       <c r="F3" s="3" t="n"/>
       <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3">
+      <c r="H3" s="3">
         <f>16.25</f>
         <v/>
       </c>
+      <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="n"/>
       <c r="N3" s="3">
-        <f>SUM(B3:M3)</f>
-        <v/>
-      </c>
-      <c r="O3" s="1" t="inlineStr">
+        <f>16.25</f>
+        <v/>
+      </c>
+      <c r="O3" s="3">
+        <f>SUM(B3,C3,D3,E3,F3,G3,H3,I3,J3,K3,L3,M3,N3,Q3)</f>
+        <v/>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
         <is>
           <t>GERCORY</t>
         </is>
+      </c>
+      <c r="Q3" s="5">
+        <f>16.25</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -3322,11 +3221,12 @@
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="n"/>
       <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3">
-        <f>SUM(B4:M4)</f>
-        <v/>
-      </c>
-      <c r="O4" s="1" t="inlineStr">
+      <c r="N4" s="3" t="n"/>
+      <c r="O4" s="3">
+        <f>SUM(B4,C4,D4,E4,F4,G4,H4,I4,J4,K4,L4,M4,N4,Q4)</f>
+        <v/>
+      </c>
+      <c r="P4" s="1" t="inlineStr">
         <is>
           <t>GERCORY</t>
         </is>
@@ -3350,11 +3250,12 @@
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="n"/>
       <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3">
-        <f>SUM(B5:M5)</f>
-        <v/>
-      </c>
-      <c r="O5" s="1" t="inlineStr">
+      <c r="N5" s="3" t="n"/>
+      <c r="O5" s="3">
+        <f>SUM(B5,C5,D5,E5,F5,G5,H5,I5,J5,K5,L5,M5,N5,Q5)</f>
+        <v/>
+      </c>
+      <c r="P5" s="1" t="inlineStr">
         <is>
           <t>GERCORY</t>
         </is>
@@ -3378,11 +3279,12 @@
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="3" t="n"/>
       <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3">
-        <f>SUM(B6:M6)</f>
-        <v/>
-      </c>
-      <c r="O6" s="1" t="inlineStr">
+      <c r="N6" s="3" t="n"/>
+      <c r="O6" s="3">
+        <f>SUM(B6,C6,D6,E6,F6,G6,H6,I6,J6,K6,L6,M6,N6,Q6)</f>
+        <v/>
+      </c>
+      <c r="P6" s="1" t="inlineStr">
         <is>
           <t>GERCORY</t>
         </is>
@@ -3406,11 +3308,12 @@
       <c r="K7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
       <c r="M7" s="3" t="n"/>
-      <c r="N7" s="3">
-        <f>SUM(B7:M7)</f>
-        <v/>
-      </c>
-      <c r="O7" s="1" t="inlineStr">
+      <c r="N7" s="3" t="n"/>
+      <c r="O7" s="3">
+        <f>SUM(B7,C7,D7,E7,F7,G7,H7,I7,J7,K7,L7,M7,N7,Q7)</f>
+        <v/>
+      </c>
+      <c r="P7" s="1" t="inlineStr">
         <is>
           <t>GERCORY</t>
         </is>
@@ -3434,11 +3337,12 @@
       <c r="K8" s="3" t="n"/>
       <c r="L8" s="3" t="n"/>
       <c r="M8" s="3" t="n"/>
-      <c r="N8" s="3">
-        <f>SUM(B8:M8)</f>
-        <v/>
-      </c>
-      <c r="O8" s="1" t="inlineStr">
+      <c r="N8" s="3" t="n"/>
+      <c r="O8" s="3">
+        <f>SUM(B8,C8,D8,E8,F8,G8,H8,I8,J8,K8,L8,M8,N8,Q8)</f>
+        <v/>
+      </c>
+      <c r="P8" s="1" t="inlineStr">
         <is>
           <t>GERCORY</t>
         </is>
@@ -3462,11 +3366,12 @@
       <c r="K9" s="3" t="n"/>
       <c r="L9" s="3" t="n"/>
       <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3">
-        <f>SUM(B9:M9)</f>
-        <v/>
-      </c>
-      <c r="O9" s="1" t="inlineStr">
+      <c r="N9" s="3" t="n"/>
+      <c r="O9" s="3">
+        <f>SUM(B9,C9,D9,E9,F9,G9,H9,I9,J9,K9,L9,M9,N9,Q9)</f>
+        <v/>
+      </c>
+      <c r="P9" s="1" t="inlineStr">
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
@@ -3484,23 +3389,31 @@
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3">
+      <c r="H10" s="3">
         <f>350.00</f>
         <v/>
       </c>
+      <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="n"/>
       <c r="L10" s="3" t="n"/>
       <c r="M10" s="3" t="n"/>
       <c r="N10" s="3">
-        <f>SUM(B10:M10)</f>
-        <v/>
-      </c>
-      <c r="O10" s="1" t="inlineStr">
+        <f>350.00</f>
+        <v/>
+      </c>
+      <c r="O10" s="3">
+        <f>SUM(B10,C10,D10,E10,F10,G10,H10,I10,J10,K10,L10,M10,N10,Q10)</f>
+        <v/>
+      </c>
+      <c r="P10" s="1" t="inlineStr">
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
+      </c>
+      <c r="Q10" s="5">
+        <f>350.00</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -3521,11 +3434,12 @@
       <c r="K11" s="3" t="n"/>
       <c r="L11" s="3" t="n"/>
       <c r="M11" s="3" t="n"/>
-      <c r="N11" s="3">
-        <f>SUM(B11:M11)</f>
-        <v/>
-      </c>
-      <c r="O11" s="1" t="inlineStr">
+      <c r="N11" s="3" t="n"/>
+      <c r="O11" s="3">
+        <f>SUM(B11,C11,D11,E11,F11,G11,H11,I11,J11,K11,L11,M11,N11,Q11)</f>
+        <v/>
+      </c>
+      <c r="P11" s="1" t="inlineStr">
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
@@ -3543,23 +3457,31 @@
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3">
+      <c r="H12" s="3">
         <f>300.00</f>
         <v/>
       </c>
+      <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
       <c r="K12" s="3" t="n"/>
       <c r="L12" s="3" t="n"/>
       <c r="M12" s="3" t="n"/>
       <c r="N12" s="3">
-        <f>SUM(B12:M12)</f>
-        <v/>
-      </c>
-      <c r="O12" s="1" t="inlineStr">
+        <f>300.00</f>
+        <v/>
+      </c>
+      <c r="O12" s="3">
+        <f>SUM(B12,C12,D12,E12,F12,G12,H12,I12,J12,K12,L12,M12,N12,Q12)</f>
+        <v/>
+      </c>
+      <c r="P12" s="1" t="inlineStr">
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
+      </c>
+      <c r="Q12" s="5">
+        <f>300.00</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -3580,11 +3502,12 @@
       <c r="K13" s="3" t="n"/>
       <c r="L13" s="3" t="n"/>
       <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3">
-        <f>SUM(B13:M13)</f>
-        <v/>
-      </c>
-      <c r="O13" s="1" t="inlineStr">
+      <c r="N13" s="3" t="n"/>
+      <c r="O13" s="3">
+        <f>SUM(B13,C13,D13,E13,F13,G13,H13,I13,J13,K13,L13,M13,N13,Q13)</f>
+        <v/>
+      </c>
+      <c r="P13" s="1" t="inlineStr">
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
@@ -3602,20 +3525,31 @@
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
+      <c r="H14" s="3">
+        <f>975.00</f>
+        <v/>
+      </c>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
       <c r="K14" s="3" t="n"/>
       <c r="L14" s="3" t="n"/>
       <c r="M14" s="3" t="n"/>
       <c r="N14" s="3">
-        <f>SUM(B14:M14)</f>
-        <v/>
-      </c>
-      <c r="O14" s="1" t="inlineStr">
+        <f>975.00</f>
+        <v/>
+      </c>
+      <c r="O14" s="3">
+        <f>SUM(B14,C14,D14,E14,F14,G14,H14,I14,J14,K14,L14,M14,N14,Q14)</f>
+        <v/>
+      </c>
+      <c r="P14" s="1" t="inlineStr">
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
+      </c>
+      <c r="Q14" s="5">
+        <f>975.00</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -3630,20 +3564,31 @@
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
+      <c r="H15" s="3">
+        <f>817.29</f>
+        <v/>
+      </c>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="3" t="n"/>
       <c r="L15" s="3" t="n"/>
       <c r="M15" s="3" t="n"/>
       <c r="N15" s="3">
-        <f>SUM(B15:M15)</f>
-        <v/>
-      </c>
-      <c r="O15" s="1" t="inlineStr">
+        <f>817.29</f>
+        <v/>
+      </c>
+      <c r="O15" s="3">
+        <f>SUM(B15,C15,D15,E15,F15,G15,H15,I15,J15,K15,L15,M15,N15,Q15)</f>
+        <v/>
+      </c>
+      <c r="P15" s="1" t="inlineStr">
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
+      </c>
+      <c r="Q15" s="5">
+        <f>817.29</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -3664,11 +3609,12 @@
       <c r="K16" s="3" t="n"/>
       <c r="L16" s="3" t="n"/>
       <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3">
-        <f>SUM(B16:M16)</f>
-        <v/>
-      </c>
-      <c r="O16" s="1" t="inlineStr">
+      <c r="N16" s="3" t="n"/>
+      <c r="O16" s="3">
+        <f>SUM(B16,C16,D16,E16,F16,G16,H16,I16,J16,K16,L16,M16,N16,Q16)</f>
+        <v/>
+      </c>
+      <c r="P16" s="1" t="inlineStr">
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
@@ -3692,11 +3638,12 @@
       <c r="K17" s="3" t="n"/>
       <c r="L17" s="3" t="n"/>
       <c r="M17" s="3" t="n"/>
-      <c r="N17" s="3">
-        <f>SUM(B17:M17)</f>
-        <v/>
-      </c>
-      <c r="O17" s="1" t="inlineStr">
+      <c r="N17" s="3" t="n"/>
+      <c r="O17" s="3">
+        <f>SUM(B17,C17,D17,E17,F17,G17,H17,I17,J17,K17,L17,M17,N17,Q17)</f>
+        <v/>
+      </c>
+      <c r="P17" s="1" t="inlineStr">
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
@@ -3720,11 +3667,12 @@
       <c r="K18" s="3" t="n"/>
       <c r="L18" s="3" t="n"/>
       <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3">
-        <f>SUM(B18:M18)</f>
-        <v/>
-      </c>
-      <c r="O18" s="1" t="inlineStr">
+      <c r="N18" s="3" t="n"/>
+      <c r="O18" s="3">
+        <f>SUM(B18,C18,D18,E18,F18,G18,H18,I18,J18,K18,L18,M18,N18,Q18)</f>
+        <v/>
+      </c>
+      <c r="P18" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
@@ -3742,23 +3690,31 @@
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3">
+      <c r="H19" s="3">
         <f>385.77+740.00</f>
         <v/>
       </c>
+      <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="n"/>
       <c r="L19" s="3" t="n"/>
       <c r="M19" s="3" t="n"/>
       <c r="N19" s="3">
-        <f>SUM(B19:M19)</f>
-        <v/>
-      </c>
-      <c r="O19" s="1" t="inlineStr">
+        <f>385.77+740.00</f>
+        <v/>
+      </c>
+      <c r="O19" s="3">
+        <f>SUM(B19,C19,D19,E19,F19,G19,H19,I19,J19,K19,L19,M19,N19,Q19)</f>
+        <v/>
+      </c>
+      <c r="P19" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
+      </c>
+      <c r="Q19" s="5">
+        <f>385.77+740.00</f>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -3773,23 +3729,31 @@
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3">
+      <c r="H20" s="3">
         <f>800.00+800.00</f>
         <v/>
       </c>
+      <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
       <c r="K20" s="3" t="n"/>
       <c r="L20" s="3" t="n"/>
       <c r="M20" s="3" t="n"/>
       <c r="N20" s="3">
-        <f>SUM(B20:M20)</f>
-        <v/>
-      </c>
-      <c r="O20" s="1" t="inlineStr">
+        <f>800.00+800.00</f>
+        <v/>
+      </c>
+      <c r="O20" s="3">
+        <f>SUM(B20,C20,D20,E20,F20,G20,H20,I20,J20,K20,L20,M20,N20,Q20)</f>
+        <v/>
+      </c>
+      <c r="P20" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
+      </c>
+      <c r="Q20" s="5">
+        <f>800.00+800.00</f>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -3804,23 +3768,31 @@
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3">
-        <f>490.00</f>
-        <v/>
-      </c>
+      <c r="H21" s="3">
+        <f>490.00+120.00</f>
+        <v/>
+      </c>
+      <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
       <c r="K21" s="3" t="n"/>
       <c r="L21" s="3" t="n"/>
       <c r="M21" s="3" t="n"/>
       <c r="N21" s="3">
-        <f>SUM(B21:M21)</f>
-        <v/>
-      </c>
-      <c r="O21" s="1" t="inlineStr">
+        <f>490.00+120.00</f>
+        <v/>
+      </c>
+      <c r="O21" s="3">
+        <f>SUM(B21,C21,D21,E21,F21,G21,H21,I21,J21,K21,L21,M21,N21,Q21)</f>
+        <v/>
+      </c>
+      <c r="P21" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
+      </c>
+      <c r="Q21" s="5">
+        <f>490.00+120.00</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -3835,23 +3807,31 @@
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3">
+      <c r="H22" s="3">
         <f>4000.00</f>
         <v/>
       </c>
+      <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
       <c r="K22" s="3" t="n"/>
       <c r="L22" s="3" t="n"/>
       <c r="M22" s="3" t="n"/>
       <c r="N22" s="3">
-        <f>SUM(B22:M22)</f>
-        <v/>
-      </c>
-      <c r="O22" s="1" t="inlineStr">
+        <f>4000.00</f>
+        <v/>
+      </c>
+      <c r="O22" s="3">
+        <f>SUM(B22,C22,D22,E22,F22,G22,H22,I22,J22,K22,L22,M22,N22,Q22)</f>
+        <v/>
+      </c>
+      <c r="P22" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
+      </c>
+      <c r="Q22" s="5">
+        <f>4000.00</f>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -3872,11 +3852,12 @@
       <c r="K23" s="3" t="n"/>
       <c r="L23" s="3" t="n"/>
       <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3">
-        <f>SUM(B23:M23)</f>
-        <v/>
-      </c>
-      <c r="O23" s="1" t="inlineStr">
+      <c r="N23" s="3" t="n"/>
+      <c r="O23" s="3">
+        <f>SUM(B23,C23,D23,E23,F23,G23,H23,I23,J23,K23,L23,M23,N23,Q23)</f>
+        <v/>
+      </c>
+      <c r="P23" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
@@ -3894,23 +3875,31 @@
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3">
+      <c r="H24" s="3">
         <f>200.00+200.00</f>
         <v/>
       </c>
+      <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
       <c r="K24" s="3" t="n"/>
       <c r="L24" s="3" t="n"/>
       <c r="M24" s="3" t="n"/>
       <c r="N24" s="3">
-        <f>SUM(B24:M24)</f>
-        <v/>
-      </c>
-      <c r="O24" s="1" t="inlineStr">
+        <f>200.00+200.00</f>
+        <v/>
+      </c>
+      <c r="O24" s="3">
+        <f>SUM(B24,C24,D24,E24,F24,G24,H24,I24,J24,K24,L24,M24,N24,Q24)</f>
+        <v/>
+      </c>
+      <c r="P24" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
+      </c>
+      <c r="Q24" s="5">
+        <f>200.00+200.00</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -3931,11 +3920,12 @@
       <c r="K25" s="3" t="n"/>
       <c r="L25" s="3" t="n"/>
       <c r="M25" s="3" t="n"/>
-      <c r="N25" s="3">
-        <f>SUM(B25:M25)</f>
-        <v/>
-      </c>
-      <c r="O25" s="1" t="inlineStr">
+      <c r="N25" s="3" t="n"/>
+      <c r="O25" s="3">
+        <f>SUM(B25,C25,D25,E25,F25,G25,H25,I25,J25,K25,L25,M25,N25,Q25)</f>
+        <v/>
+      </c>
+      <c r="P25" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
@@ -3959,11 +3949,12 @@
       <c r="K26" s="3" t="n"/>
       <c r="L26" s="3" t="n"/>
       <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3">
-        <f>SUM(B26:M26)</f>
-        <v/>
-      </c>
-      <c r="O26" s="1" t="inlineStr">
+      <c r="N26" s="3" t="n"/>
+      <c r="O26" s="3">
+        <f>SUM(B26,C26,D26,E26,F26,G26,H26,I26,J26,K26,L26,M26,N26,Q26)</f>
+        <v/>
+      </c>
+      <c r="P26" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
@@ -3981,23 +3972,31 @@
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3">
+      <c r="H27" s="3">
         <f>26.57</f>
         <v/>
       </c>
+      <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
       <c r="K27" s="3" t="n"/>
       <c r="L27" s="3" t="n"/>
       <c r="M27" s="3" t="n"/>
       <c r="N27" s="3">
-        <f>SUM(B27:M27)</f>
-        <v/>
-      </c>
-      <c r="O27" s="1" t="inlineStr">
+        <f>26.57</f>
+        <v/>
+      </c>
+      <c r="O27" s="3">
+        <f>SUM(B27,C27,D27,E27,F27,G27,H27,I27,J27,K27,L27,M27,N27,Q27)</f>
+        <v/>
+      </c>
+      <c r="P27" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
+      </c>
+      <c r="Q27" s="5">
+        <f>26.57</f>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -4018,11 +4017,12 @@
       <c r="K28" s="3" t="n"/>
       <c r="L28" s="3" t="n"/>
       <c r="M28" s="3" t="n"/>
-      <c r="N28" s="3">
-        <f>SUM(B28:M28)</f>
-        <v/>
-      </c>
-      <c r="O28" s="1" t="inlineStr">
+      <c r="N28" s="3" t="n"/>
+      <c r="O28" s="3">
+        <f>SUM(B28,C28,D28,E28,F28,G28,H28,I28,J28,K28,L28,M28,N28,Q28)</f>
+        <v/>
+      </c>
+      <c r="P28" s="1" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
@@ -4046,11 +4046,12 @@
       <c r="K29" s="3" t="n"/>
       <c r="L29" s="3" t="n"/>
       <c r="M29" s="3" t="n"/>
-      <c r="N29" s="3">
-        <f>SUM(B29:M29)</f>
-        <v/>
-      </c>
-      <c r="O29" s="1" t="inlineStr">
+      <c r="N29" s="3" t="n"/>
+      <c r="O29" s="3">
+        <f>SUM(B29,C29,D29,E29,F29,G29,H29,I29,J29,K29,L29,M29,N29,Q29)</f>
+        <v/>
+      </c>
+      <c r="P29" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
@@ -4074,11 +4075,12 @@
       <c r="K30" s="3" t="n"/>
       <c r="L30" s="3" t="n"/>
       <c r="M30" s="3" t="n"/>
-      <c r="N30" s="3">
-        <f>SUM(B30:M30)</f>
-        <v/>
-      </c>
-      <c r="O30" s="1" t="inlineStr">
+      <c r="N30" s="3" t="n"/>
+      <c r="O30" s="3">
+        <f>SUM(B30,C30,D30,E30,F30,G30,H30,I30,J30,K30,L30,M30,N30,Q30)</f>
+        <v/>
+      </c>
+      <c r="P30" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
@@ -4102,11 +4104,12 @@
       <c r="K31" s="3" t="n"/>
       <c r="L31" s="3" t="n"/>
       <c r="M31" s="3" t="n"/>
-      <c r="N31" s="3">
-        <f>SUM(B31:M31)</f>
-        <v/>
-      </c>
-      <c r="O31" s="1" t="inlineStr">
+      <c r="N31" s="3" t="n"/>
+      <c r="O31" s="3">
+        <f>SUM(B31,C31,D31,E31,F31,G31,H31,I31,J31,K31,L31,M31,N31,Q31)</f>
+        <v/>
+      </c>
+      <c r="P31" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
@@ -4124,23 +4127,31 @@
       <c r="E32" s="3" t="n"/>
       <c r="F32" s="3" t="n"/>
       <c r="G32" s="3" t="n"/>
-      <c r="H32" s="3" t="n"/>
-      <c r="I32" s="3">
+      <c r="H32" s="3">
         <f>75.40</f>
         <v/>
       </c>
+      <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
       <c r="K32" s="3" t="n"/>
       <c r="L32" s="3" t="n"/>
       <c r="M32" s="3" t="n"/>
       <c r="N32" s="3">
-        <f>SUM(B32:M32)</f>
-        <v/>
-      </c>
-      <c r="O32" s="1" t="inlineStr">
+        <f>75.40</f>
+        <v/>
+      </c>
+      <c r="O32" s="3">
+        <f>SUM(B32,C32,D32,E32,F32,G32,H32,I32,J32,K32,L32,M32,N32,Q32)</f>
+        <v/>
+      </c>
+      <c r="P32" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
+      </c>
+      <c r="Q32" s="5">
+        <f>75.40</f>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -4155,23 +4166,31 @@
       <c r="E33" s="3" t="n"/>
       <c r="F33" s="3" t="n"/>
       <c r="G33" s="3" t="n"/>
-      <c r="H33" s="3" t="n"/>
-      <c r="I33" s="3">
+      <c r="H33" s="3">
         <f>18.75</f>
         <v/>
       </c>
+      <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
       <c r="K33" s="3" t="n"/>
       <c r="L33" s="3" t="n"/>
       <c r="M33" s="3" t="n"/>
       <c r="N33" s="3">
-        <f>SUM(B33:M33)</f>
-        <v/>
-      </c>
-      <c r="O33" s="1" t="inlineStr">
+        <f>18.75</f>
+        <v/>
+      </c>
+      <c r="O33" s="3">
+        <f>SUM(B33,C33,D33,E33,F33,G33,H33,I33,J33,K33,L33,M33,N33,Q33)</f>
+        <v/>
+      </c>
+      <c r="P33" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
+      </c>
+      <c r="Q33" s="5">
+        <f>18.75</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -4192,11 +4211,12 @@
       <c r="K34" s="3" t="n"/>
       <c r="L34" s="3" t="n"/>
       <c r="M34" s="3" t="n"/>
-      <c r="N34" s="3">
-        <f>SUM(B34:M34)</f>
-        <v/>
-      </c>
-      <c r="O34" s="1" t="inlineStr">
+      <c r="N34" s="3" t="n"/>
+      <c r="O34" s="3">
+        <f>SUM(B34,C34,D34,E34,F34,G34,H34,I34,J34,K34,L34,M34,N34,Q34)</f>
+        <v/>
+      </c>
+      <c r="P34" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
@@ -4220,11 +4240,12 @@
       <c r="K35" s="3" t="n"/>
       <c r="L35" s="3" t="n"/>
       <c r="M35" s="3" t="n"/>
-      <c r="N35" s="3">
-        <f>SUM(B35:M35)</f>
-        <v/>
-      </c>
-      <c r="O35" s="1" t="inlineStr">
+      <c r="N35" s="3" t="n"/>
+      <c r="O35" s="3">
+        <f>SUM(B35,C35,D35,E35,F35,G35,H35,I35,J35,K35,L35,M35,N35,Q35)</f>
+        <v/>
+      </c>
+      <c r="P35" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
@@ -4248,11 +4269,12 @@
       <c r="K36" s="3" t="n"/>
       <c r="L36" s="3" t="n"/>
       <c r="M36" s="3" t="n"/>
-      <c r="N36" s="3">
-        <f>SUM(B36:M36)</f>
-        <v/>
-      </c>
-      <c r="O36" s="1" t="inlineStr">
+      <c r="N36" s="3" t="n"/>
+      <c r="O36" s="3">
+        <f>SUM(B36,C36,D36,E36,F36,G36,H36,I36,J36,K36,L36,M36,N36,Q36)</f>
+        <v/>
+      </c>
+      <c r="P36" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
@@ -4276,11 +4298,12 @@
       <c r="K37" s="3" t="n"/>
       <c r="L37" s="3" t="n"/>
       <c r="M37" s="3" t="n"/>
-      <c r="N37" s="3">
-        <f>SUM(B37:M37)</f>
-        <v/>
-      </c>
-      <c r="O37" s="1" t="inlineStr">
+      <c r="N37" s="3" t="n"/>
+      <c r="O37" s="3">
+        <f>SUM(B37,C37,D37,E37,F37,G37,H37,I37,J37,K37,L37,M37,N37,Q37)</f>
+        <v/>
+      </c>
+      <c r="P37" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
@@ -4298,20 +4321,31 @@
       <c r="E38" s="3" t="n"/>
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="n"/>
-      <c r="H38" s="3" t="n"/>
+      <c r="H38" s="3">
+        <f>930.52</f>
+        <v/>
+      </c>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
       <c r="K38" s="3" t="n"/>
       <c r="L38" s="3" t="n"/>
       <c r="M38" s="3" t="n"/>
       <c r="N38" s="3">
-        <f>SUM(B38:M38)</f>
-        <v/>
-      </c>
-      <c r="O38" s="1" t="inlineStr">
+        <f>930.52</f>
+        <v/>
+      </c>
+      <c r="O38" s="3">
+        <f>SUM(B38,C38,D38,E38,F38,G38,H38,I38,J38,K38,L38,M38,N38,Q38)</f>
+        <v/>
+      </c>
+      <c r="P38" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
+      </c>
+      <c r="Q38" s="5">
+        <f>930.52</f>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -4332,11 +4366,12 @@
       <c r="K39" s="3" t="n"/>
       <c r="L39" s="3" t="n"/>
       <c r="M39" s="3" t="n"/>
-      <c r="N39" s="3">
-        <f>SUM(B39:M39)</f>
-        <v/>
-      </c>
-      <c r="O39" s="1" t="inlineStr">
+      <c r="N39" s="3" t="n"/>
+      <c r="O39" s="3">
+        <f>SUM(B39,C39,D39,E39,F39,G39,H39,I39,J39,K39,L39,M39,N39,Q39)</f>
+        <v/>
+      </c>
+      <c r="P39" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
@@ -4354,23 +4389,31 @@
       <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="n"/>
       <c r="G40" s="3" t="n"/>
-      <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3">
+      <c r="H40" s="3">
         <f>1000.00+3200.00</f>
         <v/>
       </c>
+      <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
       <c r="K40" s="3" t="n"/>
       <c r="L40" s="3" t="n"/>
       <c r="M40" s="3" t="n"/>
       <c r="N40" s="3">
-        <f>SUM(B40:M40)</f>
-        <v/>
-      </c>
-      <c r="O40" s="1" t="inlineStr">
+        <f>1000.00+3200.00</f>
+        <v/>
+      </c>
+      <c r="O40" s="3">
+        <f>SUM(B40,C40,D40,E40,F40,G40,H40,I40,J40,K40,L40,M40,N40,Q40)</f>
+        <v/>
+      </c>
+      <c r="P40" s="1" t="inlineStr">
         <is>
           <t>SUPPLY</t>
         </is>
+      </c>
+      <c r="Q40" s="5">
+        <f>1000.00+3200.00</f>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -4428,10 +4471,18 @@
         <v/>
       </c>
       <c r="N41" s="3">
-        <f>SUM(B41:M41)</f>
-        <v/>
-      </c>
-      <c r="O41" s="1" t="n"/>
+        <f>SUM(N2:N40)</f>
+        <v/>
+      </c>
+      <c r="O41" s="3">
+        <f>SUM(B41,C41,D41,E41,F41,G41,H41,I41,J41,K41,L41,M41,N41,Q41)</f>
+        <v/>
+      </c>
+      <c r="P41" s="1" t="n"/>
+      <c r="Q41" s="5">
+        <f>SUM(Q2:Q40)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
lazy pudding tool commit
</commit_message>
<xml_diff>
--- a/credit_monthly_summary.xlsx
+++ b/credit_monthly_summary.xlsx
@@ -121,9 +121,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -135,6 +132,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -510,7 +510,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>CHASE #3444</t>
         </is>
@@ -535,93 +535,93 @@
       <c r="S1" s="9" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="6" t="n"/>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="n"/>
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>BEGIN BALANCE</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>CASH / CHECK DEPOSIT</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>NO1 SUSHI 88 CORKBBO ACH</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>VEOLIA WATER</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>ORANGE &amp; ROCKLAND</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>WITHDRAWAL BRANCH 0964</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>AMAZON</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>BILL PAY:VEOLIA WATER NEW Y 200045 6BU1T6KR</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>BILL PAY:ORANGE &amp; ROCKLAND 136130 6BQ1P6KR</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>INTERNET TRF TO CLIENT-ADDED TRANSFER ACCOUNT</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="L2" s="7" t="inlineStr">
         <is>
           <t>WITHDRAWAL BRANCH 0964 NEW YORK</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*NX6 SEATTLE WA</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="N2" s="7" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*9O5 SEATTLE WA</t>
         </is>
       </c>
-      <c r="O2" s="6" t="inlineStr">
+      <c r="O2" s="7" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*SB8 SEATTLE WA</t>
         </is>
       </c>
-      <c r="P2" s="6" t="inlineStr">
+      <c r="P2" s="7" t="inlineStr">
         <is>
           <t>NYS DTF PIT TAX PAYMNT</t>
         </is>
       </c>
-      <c r="Q2" s="6" t="inlineStr">
+      <c r="Q2" s="7" t="inlineStr">
         <is>
           <t>TOTAL CREDIT</t>
         </is>
       </c>
-      <c r="R2" s="6" t="inlineStr">
+      <c r="R2" s="7" t="inlineStr">
         <is>
           <t>DEBIT</t>
         </is>
       </c>
-      <c r="S2" s="6" t="inlineStr">
+      <c r="S2" s="7" t="inlineStr">
         <is>
           <t>ENDING BALANCE</t>
         </is>
@@ -633,29 +633,29 @@
           <t>AUG</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3">
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2">
         <f>SUM(C3:P3)</f>
         <v/>
       </c>
-      <c r="R3" s="3" t="n"/>
-      <c r="S3" s="3">
+      <c r="R3" s="2" t="n"/>
+      <c r="S3" s="2">
         <f>B3+Q3-R3</f>
         <v/>
       </c>
@@ -666,30 +666,30 @@
           <t>SEP</t>
         </is>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <f>S3</f>
         <v/>
       </c>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3">
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="n"/>
+      <c r="P4" s="2" t="n"/>
+      <c r="Q4" s="2">
         <f>SUM(C4:P4)</f>
         <v/>
       </c>
-      <c r="R4" s="3" t="n"/>
-      <c r="S4" s="3">
+      <c r="R4" s="2" t="n"/>
+      <c r="S4" s="2">
         <f>B4+Q4-R4</f>
         <v/>
       </c>
@@ -700,30 +700,30 @@
           <t>OCT</t>
         </is>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <f>S4</f>
         <v/>
       </c>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="3" t="n"/>
-      <c r="Q5" s="3">
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
+      <c r="O5" s="2" t="n"/>
+      <c r="P5" s="2" t="n"/>
+      <c r="Q5" s="2">
         <f>SUM(C5:P5)</f>
         <v/>
       </c>
-      <c r="R5" s="3" t="n"/>
-      <c r="S5" s="3">
+      <c r="R5" s="2" t="n"/>
+      <c r="S5" s="2">
         <f>B5+Q5-R5</f>
         <v/>
       </c>
@@ -734,30 +734,30 @@
           <t>NOV</t>
         </is>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <f>S5</f>
         <v/>
       </c>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="3" t="n"/>
-      <c r="Q6" s="3">
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
+      <c r="O6" s="2" t="n"/>
+      <c r="P6" s="2" t="n"/>
+      <c r="Q6" s="2">
         <f>SUM(C6:P6)</f>
         <v/>
       </c>
-      <c r="R6" s="3" t="n"/>
-      <c r="S6" s="3">
+      <c r="R6" s="2" t="n"/>
+      <c r="S6" s="2">
         <f>B6+Q6-R6</f>
         <v/>
       </c>
@@ -768,30 +768,30 @@
           <t>DEC</t>
         </is>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <f>S6</f>
         <v/>
       </c>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="n"/>
-      <c r="N7" s="3" t="n"/>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="3" t="n"/>
-      <c r="Q7" s="3">
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="2">
         <f>SUM(C7:P7)</f>
         <v/>
       </c>
-      <c r="R7" s="3" t="n"/>
-      <c r="S7" s="3">
+      <c r="R7" s="2" t="n"/>
+      <c r="S7" s="2">
         <f>B7+Q7-R7</f>
         <v/>
       </c>
@@ -802,30 +802,30 @@
           <t>JAN</t>
         </is>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <f>S7</f>
         <v/>
       </c>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="N8" s="3" t="n"/>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="3" t="n"/>
-      <c r="Q8" s="3">
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="n"/>
+      <c r="N8" s="2" t="n"/>
+      <c r="O8" s="2" t="n"/>
+      <c r="P8" s="2" t="n"/>
+      <c r="Q8" s="2">
         <f>SUM(C8:P8)</f>
         <v/>
       </c>
-      <c r="R8" s="3" t="n"/>
-      <c r="S8" s="3">
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2">
         <f>B8+Q8-R8</f>
         <v/>
       </c>
@@ -836,30 +836,30 @@
           <t>FEB</t>
         </is>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <f>S8</f>
         <v/>
       </c>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="3" t="n"/>
-      <c r="Q9" s="3">
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="n"/>
+      <c r="P9" s="2" t="n"/>
+      <c r="Q9" s="2">
         <f>SUM(C9:P9)</f>
         <v/>
       </c>
-      <c r="R9" s="3" t="n"/>
-      <c r="S9" s="3">
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="2">
         <f>B9+Q9-R9</f>
         <v/>
       </c>
@@ -870,30 +870,30 @@
           <t>MAR</t>
         </is>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <f>S9</f>
         <v/>
       </c>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="3" t="n"/>
-      <c r="Q10" s="3">
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2" t="n"/>
+      <c r="P10" s="2" t="n"/>
+      <c r="Q10" s="2">
         <f>SUM(C10:P10)</f>
         <v/>
       </c>
-      <c r="R10" s="3" t="n"/>
-      <c r="S10" s="3">
+      <c r="R10" s="2" t="n"/>
+      <c r="S10" s="2">
         <f>B10+Q10-R10</f>
         <v/>
       </c>
@@ -904,30 +904,30 @@
           <t>APR</t>
         </is>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <f>S10</f>
         <v/>
       </c>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
-      <c r="N11" s="3" t="n"/>
-      <c r="O11" s="3" t="n"/>
-      <c r="P11" s="3" t="n"/>
-      <c r="Q11" s="3">
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2" t="n"/>
+      <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="2">
         <f>SUM(C11:P11)</f>
         <v/>
       </c>
-      <c r="R11" s="3" t="n"/>
-      <c r="S11" s="3">
+      <c r="R11" s="2" t="n"/>
+      <c r="S11" s="2">
         <f>B11+Q11-R11</f>
         <v/>
       </c>
@@ -938,30 +938,30 @@
           <t>MAY</t>
         </is>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="2">
         <f>S11</f>
         <v/>
       </c>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
-      <c r="M12" s="3" t="n"/>
-      <c r="N12" s="3" t="n"/>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="3" t="n"/>
-      <c r="Q12" s="3">
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="n"/>
+      <c r="Q12" s="2">
         <f>SUM(C12:P12)</f>
         <v/>
       </c>
-      <c r="R12" s="3" t="n"/>
-      <c r="S12" s="3">
+      <c r="R12" s="2" t="n"/>
+      <c r="S12" s="2">
         <f>B12+Q12-R12</f>
         <v/>
       </c>
@@ -972,30 +972,30 @@
           <t>JUN</t>
         </is>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="2">
         <f>S12</f>
         <v/>
       </c>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="3" t="n"/>
-      <c r="Q13" s="3">
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2" t="n"/>
+      <c r="P13" s="2" t="n"/>
+      <c r="Q13" s="2">
         <f>SUM(C13:P13)</f>
         <v/>
       </c>
-      <c r="R13" s="3" t="n"/>
-      <c r="S13" s="3">
+      <c r="R13" s="2" t="n"/>
+      <c r="S13" s="2">
         <f>B13+Q13-R13</f>
         <v/>
       </c>
@@ -1006,30 +1006,30 @@
           <t>JUL</t>
         </is>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="2">
         <f>S13</f>
         <v/>
       </c>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="n"/>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="3" t="n"/>
-      <c r="Q14" s="3">
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="n"/>
+      <c r="P14" s="2" t="n"/>
+      <c r="Q14" s="2">
         <f>SUM(C14:P14)</f>
         <v/>
       </c>
-      <c r="R14" s="3" t="n"/>
-      <c r="S14" s="3">
+      <c r="R14" s="2" t="n"/>
+      <c r="S14" s="2">
         <f>B14+Q14-R14</f>
         <v/>
       </c>
@@ -1040,72 +1040,72 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3">
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2">
         <f>SUM(C3:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <f>SUM(D3:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="2">
         <f>SUM(E3:E14)</f>
         <v/>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="2">
         <f>SUM(F3:F14)</f>
         <v/>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="2">
         <f>SUM(G3:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="2">
         <f>SUM(H3:H14)</f>
         <v/>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="2">
         <f>SUM(I3:I14)</f>
         <v/>
       </c>
-      <c r="J15" s="3">
+      <c r="J15" s="2">
         <f>SUM(J3:J14)</f>
         <v/>
       </c>
-      <c r="K15" s="3">
+      <c r="K15" s="2">
         <f>SUM(K3:K14)</f>
         <v/>
       </c>
-      <c r="L15" s="3">
+      <c r="L15" s="2">
         <f>SUM(L3:L14)</f>
         <v/>
       </c>
-      <c r="M15" s="3">
+      <c r="M15" s="2">
         <f>SUM(M3:M14)</f>
         <v/>
       </c>
-      <c r="N15" s="3">
+      <c r="N15" s="2">
         <f>SUM(N3:N14)</f>
         <v/>
       </c>
-      <c r="O15" s="3">
+      <c r="O15" s="2">
         <f>SUM(O3:O14)</f>
         <v/>
       </c>
-      <c r="P15" s="3">
+      <c r="P15" s="2">
         <f>SUM(P3:P14)</f>
         <v/>
       </c>
-      <c r="Q15" s="3">
+      <c r="Q15" s="2">
         <f>SUM(Q3:Q14)</f>
         <v/>
       </c>
-      <c r="R15" s="3">
+      <c r="R15" s="2">
         <f>SUM(R3:R14)</f>
         <v/>
       </c>
-      <c r="S15" s="3">
+      <c r="S15" s="2">
         <f>S14</f>
         <v/>
       </c>
@@ -1135,77 +1135,77 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Merchant</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>SEP</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>DEC</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>JAN</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>FEB</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>MAR</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>APR</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>MAY</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>JUN</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>JUL</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="N1" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="O1" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
@@ -1217,19 +1217,19 @@
           <t>434 / Nys Commission</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2">
         <f>SUM(B2,C2,D2,E2,F2,G2,H2,I2,J2,K2,L2,M2)</f>
         <v/>
       </c>
@@ -1245,19 +1245,19 @@
           <t>Amazon Prime*Zh8618Uz3 Amzn.Com/Bill WA</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2">
         <f>SUM(B3,C3,D3,E3,F3,G3,H3,I3,J3,K3,L3,M3)</f>
         <v/>
       </c>
@@ -1273,19 +1273,19 @@
           <t>Amazon.Com*N22Fjseattlewa US</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2">
         <f>SUM(B4,C4,D4,E4,F4,G4,H4,I4,J4,K4,L4,M4)</f>
         <v/>
       </c>
@@ -1301,19 +1301,19 @@
           <t>Amazon.Comseattlewa US</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3">
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2">
         <f>SUM(B5,C5,D5,E5,F5,G5,H5,I5,J5,K5,L5,M5)</f>
         <v/>
       </c>
@@ -1329,19 +1329,19 @@
           <t>Amex Epayment ACH Pmt</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3">
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2">
         <f>SUM(B6,C6,D6,E6,F6,G6,H6,I6,J6,K6,L6,M6)</f>
         <v/>
       </c>
@@ -1357,19 +1357,19 @@
           <t>Arrow Bank Na Web Pmt</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="n"/>
-      <c r="N7" s="3">
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2">
         <f>SUM(B7,C7,D7,E7,F7,G7,H7,I7,J7,K7,L7,M7)</f>
         <v/>
       </c>
@@ -1385,19 +1385,19 @@
           <t>Bill Pay:Associated Mutual 210061 Ubq1P6Kr</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="N8" s="3">
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="n"/>
+      <c r="N8" s="2">
         <f>SUM(B8,C8,D8,E8,F8,G8,H8,I8,J8,K8,L8,M8)</f>
         <v/>
       </c>
@@ -1413,19 +1413,19 @@
           <t>Bill Pay:New York State Ins 237224 4Bq1P6Kr</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3">
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2">
         <f>SUM(B9,C9,D9,E9,F9,G9,H9,I9,J9,K9,L9,M9)</f>
         <v/>
       </c>
@@ -1441,19 +1441,19 @@
           <t>Bill Pay:Orange &amp; Rockland 136130 6Bq1P6Kr</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="N10" s="3">
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="2">
         <f>SUM(B10,C10,D10,E10,F10,G10,H10,I10,J10,K10,L10,M10)</f>
         <v/>
       </c>
@@ -1469,19 +1469,19 @@
           <t>Bill Pay:Orange &amp; Rockland 879293 5Bq1P6Kr</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
-      <c r="N11" s="3">
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2">
         <f>SUM(B11,C11,D11,E11,F11,G11,H11,I11,J11,K11,L11,M11)</f>
         <v/>
       </c>
@@ -1497,19 +1497,19 @@
           <t>Bill Pay:Veolia Water New Y 200045 6Bu1T6Kr</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
-      <c r="M12" s="3" t="n"/>
-      <c r="N12" s="3">
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="2">
         <f>SUM(B12,C12,D12,E12,F12,G12,H12,I12,J12,K12,L12,M12)</f>
         <v/>
       </c>
@@ -1525,19 +1525,19 @@
           <t>Bill Pay:Veolia Water New Y 200054 Hbu1T6Kr</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3">
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2">
         <f>SUM(B13,C13,D13,E13,F13,G13,H13,I13,J13,K13,L13,M13)</f>
         <v/>
       </c>
@@ -1553,19 +1553,19 @@
           <t>Citi Card Onlinepayment</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3">
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2">
         <f>SUM(B14,C14,D14,E14,F14,G14,H14,I14,J14,K14,L14,M14)</f>
         <v/>
       </c>
@@ -1581,19 +1581,19 @@
           <t>Credit One Bank Payment</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3">
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n"/>
+      <c r="M15" s="2" t="n"/>
+      <c r="N15" s="2">
         <f>SUM(B15,C15,D15,E15,F15,G15,H15,I15,J15,K15,L15,M15)</f>
         <v/>
       </c>
@@ -1609,19 +1609,19 @@
           <t>Discover Bank Net/Mobile</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="3" t="n"/>
-      <c r="L16" s="3" t="n"/>
-      <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3">
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n"/>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2">
         <f>SUM(B16,C16,D16,E16,F16,G16,H16,I16,J16,K16,L16,M16)</f>
         <v/>
       </c>
@@ -1637,19 +1637,19 @@
           <t>FIVE GUYS 1522 QSR 000001522 TULSA OK</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
-      <c r="L17" s="3" t="n"/>
-      <c r="M17" s="3" t="n"/>
-      <c r="N17" s="3">
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="2">
         <f>SUM(B17,C17,D17,E17,F17,G17,H17,I17,J17,K17,L17,M17)</f>
         <v/>
       </c>
@@ -1665,19 +1665,19 @@
           <t>Huntington Banksil Payment</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
-      <c r="L18" s="3" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3">
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n"/>
+      <c r="M18" s="2" t="n"/>
+      <c r="N18" s="2">
         <f>SUM(B18,C18,D18,E18,F18,G18,H18,I18,J18,K18,L18,M18)</f>
         <v/>
       </c>
@@ -1693,19 +1693,19 @@
           <t>Internet Trf To Client-Added Transfer Account</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="n"/>
-      <c r="M19" s="3" t="n"/>
-      <c r="N19" s="3">
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="2">
         <f>SUM(B19,C19,D19,E19,F19,G19,H19,I19,J19,K19,L19,M19)</f>
         <v/>
       </c>
@@ -1721,19 +1721,19 @@
           <t>Irs Usataxpymt</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="3" t="n"/>
-      <c r="L20" s="3" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="N20" s="3">
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="2">
         <f>SUM(B20,C20,D20,E20,F20,G20,H20,I20,J20,K20,L20,M20)</f>
         <v/>
       </c>
@@ -1749,19 +1749,19 @@
           <t>Kindercare Portland OR</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
-      <c r="M21" s="3" t="n"/>
-      <c r="N21" s="3">
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="n"/>
+      <c r="M21" s="2" t="n"/>
+      <c r="N21" s="2">
         <f>SUM(B21,C21,D21,E21,F21,G21,H21,I21,J21,K21,L21,M21)</f>
         <v/>
       </c>
@@ -1777,19 +1777,19 @@
           <t>No1 Sushi 88 Corkbbo ACH</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3">
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="2">
         <f>SUM(B22,C22,D22,E22,F22,G22,H22,I22,J22,K22,L22,M22)</f>
         <v/>
       </c>
@@ -1805,19 +1805,19 @@
           <t>NORDSTROM DIRECT http://shop.nordstrom WA</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3">
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="n"/>
+      <c r="N23" s="2">
         <f>SUM(B23,C23,D23,E23,F23,G23,H23,I23,J23,K23,L23,M23)</f>
         <v/>
       </c>
@@ -1833,19 +1833,19 @@
           <t>Nys Dtf Pit Tax Paymnt</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3">
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
+      <c r="M24" s="2" t="n"/>
+      <c r="N24" s="2">
         <f>SUM(B24,C24,D24,E24,F24,G24,H24,I24,J24,K24,L24,M24)</f>
         <v/>
       </c>
@@ -1861,19 +1861,19 @@
           <t>PANDA EXPRESS TACOMA WA</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
-      <c r="L25" s="3" t="n"/>
-      <c r="M25" s="3" t="n"/>
-      <c r="N25" s="3">
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
+      <c r="M25" s="2" t="n"/>
+      <c r="N25" s="2">
         <f>SUM(B25,C25,D25,E25,F25,G25,H25,I25,J25,K25,L25,M25)</f>
         <v/>
       </c>
@@ -1889,19 +1889,19 @@
           <t>Paypal Inst Xfer</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="n"/>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3">
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="n"/>
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2">
         <f>SUM(B26,C26,D26,E26,F26,G26,H26,I26,J26,K26,L26,M26)</f>
         <v/>
       </c>
@@ -1917,19 +1917,19 @@
           <t>POS Mac Amazon.Com*9O5 Seattle WA</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="3" t="n"/>
-      <c r="L27" s="3" t="n"/>
-      <c r="M27" s="3" t="n"/>
-      <c r="N27" s="3">
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
+      <c r="L27" s="2" t="n"/>
+      <c r="M27" s="2" t="n"/>
+      <c r="N27" s="2">
         <f>SUM(B27,C27,D27,E27,F27,G27,H27,I27,J27,K27,L27,M27)</f>
         <v/>
       </c>
@@ -1945,19 +1945,19 @@
           <t>POS Mac Amazon.Com*Au5 Seattle WA</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="n"/>
-      <c r="K28" s="3" t="n"/>
-      <c r="L28" s="3" t="n"/>
-      <c r="M28" s="3" t="n"/>
-      <c r="N28" s="3">
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="n"/>
+      <c r="M28" s="2" t="n"/>
+      <c r="N28" s="2">
         <f>SUM(B28,C28,D28,E28,F28,G28,H28,I28,J28,K28,L28,M28)</f>
         <v/>
       </c>
@@ -1973,19 +1973,19 @@
           <t>POS Mac Amazon.Com*Bq9 Seattle WA</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="3" t="n"/>
-      <c r="K29" s="3" t="n"/>
-      <c r="L29" s="3" t="n"/>
-      <c r="M29" s="3" t="n"/>
-      <c r="N29" s="3">
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="2" t="n"/>
+      <c r="M29" s="2" t="n"/>
+      <c r="N29" s="2">
         <f>SUM(B29,C29,D29,E29,F29,G29,H29,I29,J29,K29,L29,M29)</f>
         <v/>
       </c>
@@ -2001,19 +2001,19 @@
           <t>POS Mac Amazon.Com*Ge2 Seattle WA</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="3" t="n"/>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="3" t="n"/>
-      <c r="K30" s="3" t="n"/>
-      <c r="L30" s="3" t="n"/>
-      <c r="M30" s="3" t="n"/>
-      <c r="N30" s="3">
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="n"/>
+      <c r="M30" s="2" t="n"/>
+      <c r="N30" s="2">
         <f>SUM(B30,C30,D30,E30,F30,G30,H30,I30,J30,K30,L30,M30)</f>
         <v/>
       </c>
@@ -2029,19 +2029,19 @@
           <t>POS Mac Amazon.Com*Mz5 Seattle WA</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
-      <c r="F31" s="3" t="n"/>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="3" t="n"/>
-      <c r="I31" s="3" t="n"/>
-      <c r="J31" s="3" t="n"/>
-      <c r="K31" s="3" t="n"/>
-      <c r="L31" s="3" t="n"/>
-      <c r="M31" s="3" t="n"/>
-      <c r="N31" s="3">
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="n"/>
+      <c r="M31" s="2" t="n"/>
+      <c r="N31" s="2">
         <f>SUM(B31,C31,D31,E31,F31,G31,H31,I31,J31,K31,L31,M31)</f>
         <v/>
       </c>
@@ -2057,19 +2057,19 @@
           <t>POS Mac Amazon.Com*Nx6 Seattle WA</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n"/>
-      <c r="C32" s="3" t="n"/>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="3" t="n"/>
-      <c r="F32" s="3" t="n"/>
-      <c r="G32" s="3" t="n"/>
-      <c r="H32" s="3" t="n"/>
-      <c r="I32" s="3" t="n"/>
-      <c r="J32" s="3" t="n"/>
-      <c r="K32" s="3" t="n"/>
-      <c r="L32" s="3" t="n"/>
-      <c r="M32" s="3" t="n"/>
-      <c r="N32" s="3">
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n"/>
+      <c r="M32" s="2" t="n"/>
+      <c r="N32" s="2">
         <f>SUM(B32,C32,D32,E32,F32,G32,H32,I32,J32,K32,L32,M32)</f>
         <v/>
       </c>
@@ -2085,19 +2085,19 @@
           <t>POS Mac Amazon.Com*Sb8 Seattle WA</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n"/>
-      <c r="G33" s="3" t="n"/>
-      <c r="H33" s="3" t="n"/>
-      <c r="I33" s="3" t="n"/>
-      <c r="J33" s="3" t="n"/>
-      <c r="K33" s="3" t="n"/>
-      <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="n"/>
-      <c r="N33" s="3">
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="n"/>
+      <c r="M33" s="2" t="n"/>
+      <c r="N33" s="2">
         <f>SUM(B33,C33,D33,E33,F33,G33,H33,I33,J33,K33,L33,M33)</f>
         <v/>
       </c>
@@ -2113,19 +2113,19 @@
           <t>POS Mac Amazon.Com*TN0 Seattle WA</t>
         </is>
       </c>
-      <c r="B34" s="3" t="n"/>
-      <c r="C34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34" s="3" t="n"/>
-      <c r="G34" s="3" t="n"/>
-      <c r="H34" s="3" t="n"/>
-      <c r="I34" s="3" t="n"/>
-      <c r="J34" s="3" t="n"/>
-      <c r="K34" s="3" t="n"/>
-      <c r="L34" s="3" t="n"/>
-      <c r="M34" s="3" t="n"/>
-      <c r="N34" s="3">
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="2" t="n"/>
+      <c r="L34" s="2" t="n"/>
+      <c r="M34" s="2" t="n"/>
+      <c r="N34" s="2">
         <f>SUM(B34,C34,D34,E34,F34,G34,H34,I34,J34,K34,L34,M34)</f>
         <v/>
       </c>
@@ -2141,19 +2141,19 @@
           <t>POS Mac Amazon.Com*V25 Seattle WA</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n"/>
-      <c r="J35" s="3" t="n"/>
-      <c r="K35" s="3" t="n"/>
-      <c r="L35" s="3" t="n"/>
-      <c r="M35" s="3" t="n"/>
-      <c r="N35" s="3">
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="n"/>
+      <c r="M35" s="2" t="n"/>
+      <c r="N35" s="2">
         <f>SUM(B35,C35,D35,E35,F35,G35,H35,I35,J35,K35,L35,M35)</f>
         <v/>
       </c>
@@ -2169,19 +2169,19 @@
           <t>POS Mac Amazon.Com*Yr6 Seattle WA</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="n"/>
-      <c r="G36" s="3" t="n"/>
-      <c r="H36" s="3" t="n"/>
-      <c r="I36" s="3" t="n"/>
-      <c r="J36" s="3" t="n"/>
-      <c r="K36" s="3" t="n"/>
-      <c r="L36" s="3" t="n"/>
-      <c r="M36" s="3" t="n"/>
-      <c r="N36" s="3">
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="n"/>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="n"/>
+      <c r="M36" s="2" t="n"/>
+      <c r="N36" s="2">
         <f>SUM(B36,C36,D36,E36,F36,G36,H36,I36,J36,K36,L36,M36)</f>
         <v/>
       </c>
@@ -2197,19 +2197,19 @@
           <t>POS Mac Amazon.Com*Za2 Seattle WA</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n"/>
-      <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
-      <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
-      <c r="H37" s="3" t="n"/>
-      <c r="I37" s="3" t="n"/>
-      <c r="J37" s="3" t="n"/>
-      <c r="K37" s="3" t="n"/>
-      <c r="L37" s="3" t="n"/>
-      <c r="M37" s="3" t="n"/>
-      <c r="N37" s="3">
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
+      <c r="M37" s="2" t="n"/>
+      <c r="N37" s="2">
         <f>SUM(B37,C37,D37,E37,F37,G37,H37,I37,J37,K37,L37,M37)</f>
         <v/>
       </c>
@@ -2225,19 +2225,19 @@
           <t>Prog Casualty Ins Prem</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n"/>
-      <c r="C38" s="3" t="n"/>
-      <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="n"/>
-      <c r="F38" s="3" t="n"/>
-      <c r="G38" s="3" t="n"/>
-      <c r="H38" s="3" t="n"/>
-      <c r="I38" s="3" t="n"/>
-      <c r="J38" s="3" t="n"/>
-      <c r="K38" s="3" t="n"/>
-      <c r="L38" s="3" t="n"/>
-      <c r="M38" s="3" t="n"/>
-      <c r="N38" s="3">
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="n"/>
+      <c r="M38" s="2" t="n"/>
+      <c r="N38" s="2">
         <f>SUM(B38,C38,D38,E38,F38,G38,H38,I38,J38,K38,L38,M38)</f>
         <v/>
       </c>
@@ -2253,19 +2253,19 @@
           <t>WHOLEFDS CHB #10588 000010588 UNIVERSITY PL WA</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n"/>
-      <c r="C39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
-      <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
-      <c r="J39" s="3" t="n"/>
-      <c r="K39" s="3" t="n"/>
-      <c r="L39" s="3" t="n"/>
-      <c r="M39" s="3" t="n"/>
-      <c r="N39" s="3">
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="n"/>
+      <c r="L39" s="2" t="n"/>
+      <c r="M39" s="2" t="n"/>
+      <c r="N39" s="2">
         <f>SUM(B39,C39,D39,E39,F39,G39,H39,I39,J39,K39,L39,M39)</f>
         <v/>
       </c>
@@ -2281,19 +2281,19 @@
           <t>Withdrawal Branch 0964 New York</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="n"/>
-      <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="n"/>
-      <c r="J40" s="3" t="n"/>
-      <c r="K40" s="3" t="n"/>
-      <c r="L40" s="3" t="n"/>
-      <c r="M40" s="3" t="n"/>
-      <c r="N40" s="3">
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
+      <c r="L40" s="2" t="n"/>
+      <c r="M40" s="2" t="n"/>
+      <c r="N40" s="2">
         <f>SUM(B40,C40,D40,E40,F40,G40,H40,I40,J40,K40,L40,M40)</f>
         <v/>
       </c>
@@ -2309,19 +2309,19 @@
           <t>discover Bank Net/Mobile</t>
         </is>
       </c>
-      <c r="B41" s="3" t="n"/>
-      <c r="C41" s="3" t="n"/>
-      <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="n"/>
-      <c r="G41" s="3" t="n"/>
-      <c r="H41" s="3" t="n"/>
-      <c r="I41" s="3" t="n"/>
-      <c r="J41" s="3" t="n"/>
-      <c r="K41" s="3" t="n"/>
-      <c r="L41" s="3" t="n"/>
-      <c r="M41" s="3" t="n"/>
-      <c r="N41" s="3">
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="2" t="n"/>
+      <c r="K41" s="2" t="n"/>
+      <c r="L41" s="2" t="n"/>
+      <c r="M41" s="2" t="n"/>
+      <c r="N41" s="2">
         <f>SUM(B41,C41,D41,E41,F41,G41,H41,I41,J41,K41,L41,M41)</f>
         <v/>
       </c>
@@ -2333,55 +2333,55 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B42" s="5">
+      <c r="B42" s="4">
         <f>SUM(B2:B41)</f>
         <v/>
       </c>
-      <c r="C42" s="5">
+      <c r="C42" s="4">
         <f>SUM(C2:C41)</f>
         <v/>
       </c>
-      <c r="D42" s="5">
+      <c r="D42" s="4">
         <f>SUM(D2:D41)</f>
         <v/>
       </c>
-      <c r="E42" s="5">
+      <c r="E42" s="4">
         <f>SUM(E2:E41)</f>
         <v/>
       </c>
-      <c r="F42" s="5">
+      <c r="F42" s="4">
         <f>SUM(F2:F41)</f>
         <v/>
       </c>
-      <c r="G42" s="5">
+      <c r="G42" s="4">
         <f>SUM(G2:G41)</f>
         <v/>
       </c>
-      <c r="H42" s="5">
+      <c r="H42" s="4">
         <f>SUM(H2:H41)</f>
         <v/>
       </c>
-      <c r="I42" s="5">
+      <c r="I42" s="4">
         <f>SUM(I2:I41)</f>
         <v/>
       </c>
-      <c r="J42" s="5">
+      <c r="J42" s="4">
         <f>SUM(J2:J41)</f>
         <v/>
       </c>
-      <c r="K42" s="5">
+      <c r="K42" s="4">
         <f>SUM(K2:K41)</f>
         <v/>
       </c>
-      <c r="L42" s="5">
+      <c r="L42" s="4">
         <f>SUM(L2:L41)</f>
         <v/>
       </c>
-      <c r="M42" s="5">
+      <c r="M42" s="4">
         <f>SUM(M2:M41)</f>
         <v/>
       </c>
-      <c r="N42" s="5">
+      <c r="N42" s="4">
         <f>SUM(B42,C42,D42,E42,F42,G42,H42,I42,J42,K42,L42,M42)</f>
         <v/>
       </c>
@@ -2424,7 +2424,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="n"/>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>CHASE #3444</t>
         </is>
@@ -2448,93 +2448,93 @@
       <c r="S1" s="1" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="n"/>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="n"/>
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>BEGIN BALANCE</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>CASH / CHECK DEPOSIT</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>NO1 SUSHI 88 CORKBBO ACH</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>VEOLIA WATER</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>ORANGE &amp; ROCKLAND</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>WITHDRAWAL BRANCH 0964</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>AMAZON</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>BILL PAY:VEOLIA WATER NEW Y 200045 6BU1T6KR</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>BILL PAY:ORANGE &amp; ROCKLAND 136130 6BQ1P6KR</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>INTERNET TRF TO CLIENT-ADDED TRANSFER ACCOUNT</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr">
+      <c r="L2" s="7" t="inlineStr">
         <is>
           <t>WITHDRAWAL BRANCH 0964 NEW YORK</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
+      <c r="M2" s="7" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*NX6 SEATTLE WA</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="N2" s="7" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*9O5 SEATTLE WA</t>
         </is>
       </c>
-      <c r="O2" s="6" t="inlineStr">
+      <c r="O2" s="7" t="inlineStr">
         <is>
           <t>POS MAC AMAZON.COM*SB8 SEATTLE WA</t>
         </is>
       </c>
-      <c r="P2" s="6" t="inlineStr">
+      <c r="P2" s="7" t="inlineStr">
         <is>
           <t>NYS DTF PIT TAX PAYMNT</t>
         </is>
       </c>
-      <c r="Q2" s="6" t="inlineStr">
+      <c r="Q2" s="7" t="inlineStr">
         <is>
           <t>TOTAL CREDIT</t>
         </is>
       </c>
-      <c r="R2" s="6" t="inlineStr">
+      <c r="R2" s="7" t="inlineStr">
         <is>
           <t>DEBIT</t>
         </is>
       </c>
-      <c r="S2" s="6" t="inlineStr">
+      <c r="S2" s="7" t="inlineStr">
         <is>
           <t>ENDING BALANCE</t>
         </is>
@@ -2546,29 +2546,29 @@
           <t>AUG</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3">
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2">
         <f>SUM(C3:P3)</f>
         <v/>
       </c>
-      <c r="R3" s="3" t="n"/>
-      <c r="S3" s="3">
+      <c r="R3" s="2" t="n"/>
+      <c r="S3" s="2">
         <f>B3+Q3-R3</f>
         <v/>
       </c>
@@ -2579,30 +2579,30 @@
           <t>SEP</t>
         </is>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <f>S3</f>
         <v/>
       </c>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3">
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="n"/>
+      <c r="P4" s="2" t="n"/>
+      <c r="Q4" s="2">
         <f>SUM(C4:P4)</f>
         <v/>
       </c>
-      <c r="R4" s="3" t="n"/>
-      <c r="S4" s="3">
+      <c r="R4" s="2" t="n"/>
+      <c r="S4" s="2">
         <f>B4+Q4-R4</f>
         <v/>
       </c>
@@ -2613,30 +2613,30 @@
           <t>OCT</t>
         </is>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <f>S4</f>
         <v/>
       </c>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="3" t="n"/>
-      <c r="Q5" s="3">
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
+      <c r="O5" s="2" t="n"/>
+      <c r="P5" s="2" t="n"/>
+      <c r="Q5" s="2">
         <f>SUM(C5:P5)</f>
         <v/>
       </c>
-      <c r="R5" s="3" t="n"/>
-      <c r="S5" s="3">
+      <c r="R5" s="2" t="n"/>
+      <c r="S5" s="2">
         <f>B5+Q5-R5</f>
         <v/>
       </c>
@@ -2647,30 +2647,30 @@
           <t>NOV</t>
         </is>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <f>S5</f>
         <v/>
       </c>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="3" t="n"/>
-      <c r="Q6" s="3">
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
+      <c r="O6" s="2" t="n"/>
+      <c r="P6" s="2" t="n"/>
+      <c r="Q6" s="2">
         <f>SUM(C6:P6)</f>
         <v/>
       </c>
-      <c r="R6" s="3" t="n"/>
-      <c r="S6" s="3">
+      <c r="R6" s="2" t="n"/>
+      <c r="S6" s="2">
         <f>B6+Q6-R6</f>
         <v/>
       </c>
@@ -2681,30 +2681,30 @@
           <t>DEC</t>
         </is>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <f>S6</f>
         <v/>
       </c>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="n"/>
-      <c r="N7" s="3" t="n"/>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="3" t="n"/>
-      <c r="Q7" s="3">
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="2">
         <f>SUM(C7:P7)</f>
         <v/>
       </c>
-      <c r="R7" s="3" t="n"/>
-      <c r="S7" s="3">
+      <c r="R7" s="2" t="n"/>
+      <c r="S7" s="2">
         <f>B7+Q7-R7</f>
         <v/>
       </c>
@@ -2715,30 +2715,30 @@
           <t>JAN</t>
         </is>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <f>S7</f>
         <v/>
       </c>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="N8" s="3" t="n"/>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="3" t="n"/>
-      <c r="Q8" s="3">
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="n"/>
+      <c r="N8" s="2" t="n"/>
+      <c r="O8" s="2" t="n"/>
+      <c r="P8" s="2" t="n"/>
+      <c r="Q8" s="2">
         <f>SUM(C8:P8)</f>
         <v/>
       </c>
-      <c r="R8" s="3" t="n"/>
-      <c r="S8" s="3">
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2">
         <f>B8+Q8-R8</f>
         <v/>
       </c>
@@ -2749,30 +2749,30 @@
           <t>FEB</t>
         </is>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <f>S8</f>
         <v/>
       </c>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="3" t="n"/>
-      <c r="Q9" s="3">
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="n"/>
+      <c r="P9" s="2" t="n"/>
+      <c r="Q9" s="2">
         <f>SUM(C9:P9)</f>
         <v/>
       </c>
-      <c r="R9" s="3" t="n"/>
-      <c r="S9" s="3">
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="2">
         <f>B9+Q9-R9</f>
         <v/>
       </c>
@@ -2783,30 +2783,30 @@
           <t>MAR</t>
         </is>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <f>S9</f>
         <v/>
       </c>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="3" t="n"/>
-      <c r="Q10" s="3">
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2" t="n"/>
+      <c r="P10" s="2" t="n"/>
+      <c r="Q10" s="2">
         <f>SUM(C10:P10)</f>
         <v/>
       </c>
-      <c r="R10" s="3" t="n"/>
-      <c r="S10" s="3">
+      <c r="R10" s="2" t="n"/>
+      <c r="S10" s="2">
         <f>B10+Q10-R10</f>
         <v/>
       </c>
@@ -2817,30 +2817,30 @@
           <t>APR</t>
         </is>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <f>S10</f>
         <v/>
       </c>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
-      <c r="N11" s="3" t="n"/>
-      <c r="O11" s="3" t="n"/>
-      <c r="P11" s="3" t="n"/>
-      <c r="Q11" s="3">
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2" t="n"/>
+      <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="2">
         <f>SUM(C11:P11)</f>
         <v/>
       </c>
-      <c r="R11" s="3" t="n"/>
-      <c r="S11" s="3">
+      <c r="R11" s="2" t="n"/>
+      <c r="S11" s="2">
         <f>B11+Q11-R11</f>
         <v/>
       </c>
@@ -2851,30 +2851,30 @@
           <t>MAY</t>
         </is>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="2">
         <f>S11</f>
         <v/>
       </c>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
-      <c r="M12" s="3" t="n"/>
-      <c r="N12" s="3" t="n"/>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="3" t="n"/>
-      <c r="Q12" s="3">
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="n"/>
+      <c r="Q12" s="2">
         <f>SUM(C12:P12)</f>
         <v/>
       </c>
-      <c r="R12" s="3" t="n"/>
-      <c r="S12" s="3">
+      <c r="R12" s="2" t="n"/>
+      <c r="S12" s="2">
         <f>B12+Q12-R12</f>
         <v/>
       </c>
@@ -2885,30 +2885,30 @@
           <t>JUN</t>
         </is>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="2">
         <f>S12</f>
         <v/>
       </c>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="3" t="n"/>
-      <c r="Q13" s="3">
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2" t="n"/>
+      <c r="P13" s="2" t="n"/>
+      <c r="Q13" s="2">
         <f>SUM(C13:P13)</f>
         <v/>
       </c>
-      <c r="R13" s="3" t="n"/>
-      <c r="S13" s="3">
+      <c r="R13" s="2" t="n"/>
+      <c r="S13" s="2">
         <f>B13+Q13-R13</f>
         <v/>
       </c>
@@ -2919,30 +2919,30 @@
           <t>JUL</t>
         </is>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="2">
         <f>S13</f>
         <v/>
       </c>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="n"/>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="3" t="n"/>
-      <c r="Q14" s="3">
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="n"/>
+      <c r="P14" s="2" t="n"/>
+      <c r="Q14" s="2">
         <f>SUM(C14:P14)</f>
         <v/>
       </c>
-      <c r="R14" s="3" t="n"/>
-      <c r="S14" s="3">
+      <c r="R14" s="2" t="n"/>
+      <c r="S14" s="2">
         <f>B14+Q14-R14</f>
         <v/>
       </c>
@@ -2953,72 +2953,72 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3">
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2">
         <f>SUM(C3:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="2">
         <f>SUM(D3:D14)</f>
         <v/>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="2">
         <f>SUM(E3:E14)</f>
         <v/>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="2">
         <f>SUM(F3:F14)</f>
         <v/>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="2">
         <f>SUM(G3:G14)</f>
         <v/>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="2">
         <f>SUM(H3:H14)</f>
         <v/>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="2">
         <f>SUM(I3:I14)</f>
         <v/>
       </c>
-      <c r="J15" s="3">
+      <c r="J15" s="2">
         <f>SUM(J3:J14)</f>
         <v/>
       </c>
-      <c r="K15" s="3">
+      <c r="K15" s="2">
         <f>SUM(K3:K14)</f>
         <v/>
       </c>
-      <c r="L15" s="3">
+      <c r="L15" s="2">
         <f>SUM(L3:L14)</f>
         <v/>
       </c>
-      <c r="M15" s="3">
+      <c r="M15" s="2">
         <f>SUM(M3:M14)</f>
         <v/>
       </c>
-      <c r="N15" s="3">
+      <c r="N15" s="2">
         <f>SUM(N3:N14)</f>
         <v/>
       </c>
-      <c r="O15" s="3">
+      <c r="O15" s="2">
         <f>SUM(O3:O14)</f>
         <v/>
       </c>
-      <c r="P15" s="3">
+      <c r="P15" s="2">
         <f>SUM(P3:P14)</f>
         <v/>
       </c>
-      <c r="Q15" s="3">
+      <c r="Q15" s="2">
         <f>SUM(Q3:Q14)</f>
         <v/>
       </c>
-      <c r="R15" s="3">
+      <c r="R15" s="2">
         <f>SUM(R3:R14)</f>
         <v/>
       </c>
-      <c r="S15" s="3">
+      <c r="S15" s="2">
         <f>S14</f>
         <v/>
       </c>
@@ -3053,85 +3053,85 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Merchant</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>AUG</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>SEP</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>OCT</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>NOV</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>DEC</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>JAN</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>FEB</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>MAR</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>APR</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>MAY</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>JUN</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>JUL</t>
         </is>
       </c>
-      <c r="N1" s="4" t="n">
+      <c r="N1" s="3" t="n">
         <v>46234</v>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="O1" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="P1" s="6" t="inlineStr">
+      <c r="P1" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="Q1" s="7" t="n">
+      <c r="Q1" s="6" t="n">
         <v>46240</v>
       </c>
     </row>
@@ -3141,20 +3141,20 @@
           <t>434 / Nys Commission</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3">
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2">
         <f>SUM(B2,C2,D2,E2,F2,G2,H2,I2,J2,K2,L2,M2,N2,Q2)</f>
         <v/>
       </c>
@@ -3170,26 +3170,20 @@
           <t>Amazon Prime*Zh8618Uz3 Amzn.Com/Bill WA</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3">
-        <f>16.25</f>
-        <v/>
-      </c>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3">
-        <f>16.25</f>
-        <v/>
-      </c>
-      <c r="O3" s="3">
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2">
         <f>SUM(B3,C3,D3,E3,F3,G3,H3,I3,J3,K3,L3,M3,N3,Q3)</f>
         <v/>
       </c>
@@ -3197,10 +3191,6 @@
         <is>
           <t>GERCORY</t>
         </is>
-      </c>
-      <c r="Q3" s="5">
-        <f>16.25</f>
-        <v/>
       </c>
     </row>
     <row r="4">
@@ -3209,20 +3199,20 @@
           <t>Amazon.Com*N22Fjseattlewa US</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3">
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2">
         <f>SUM(B4,C4,D4,E4,F4,G4,H4,I4,J4,K4,L4,M4,N4,Q4)</f>
         <v/>
       </c>
@@ -3238,20 +3228,20 @@
           <t>Amazon.Comseattlewa US</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3">
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
+      <c r="O5" s="2">
         <f>SUM(B5,C5,D5,E5,F5,G5,H5,I5,J5,K5,L5,M5,N5,Q5)</f>
         <v/>
       </c>
@@ -3267,20 +3257,20 @@
           <t>Amex Epayment ACH Pmt</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3">
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
+      <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
+      <c r="O6" s="2">
         <f>SUM(B6,C6,D6,E6,F6,G6,H6,I6,J6,K6,L6,M6,N6,Q6)</f>
         <v/>
       </c>
@@ -3296,20 +3286,20 @@
           <t>Arrow Bank Na Web Pmt</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="n"/>
-      <c r="N7" s="3" t="n"/>
-      <c r="O7" s="3">
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2">
         <f>SUM(B7,C7,D7,E7,F7,G7,H7,I7,J7,K7,L7,M7,N7,Q7)</f>
         <v/>
       </c>
@@ -3325,20 +3315,20 @@
           <t>Bill Pay:Associated Mutual 210061 Ubq1P6Kr</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="N8" s="3" t="n"/>
-      <c r="O8" s="3">
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="n"/>
+      <c r="N8" s="2" t="n"/>
+      <c r="O8" s="2">
         <f>SUM(B8,C8,D8,E8,F8,G8,H8,I8,J8,K8,L8,M8,N8,Q8)</f>
         <v/>
       </c>
@@ -3354,20 +3344,20 @@
           <t>Bill Pay:New York State Ins 237224 4Bq1P6Kr</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3">
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2">
         <f>SUM(B9,C9,D9,E9,F9,G9,H9,I9,J9,K9,L9,M9,N9,Q9)</f>
         <v/>
       </c>
@@ -3383,26 +3373,20 @@
           <t>Bill Pay:Orange &amp; Rockland 136130 6Bq1P6Kr</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3">
-        <f>350.00</f>
-        <v/>
-      </c>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="N10" s="3">
-        <f>350.00</f>
-        <v/>
-      </c>
-      <c r="O10" s="3">
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2">
         <f>SUM(B10,C10,D10,E10,F10,G10,H10,I10,J10,K10,L10,M10,N10,Q10)</f>
         <v/>
       </c>
@@ -3410,10 +3394,6 @@
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
-      </c>
-      <c r="Q10" s="5">
-        <f>350.00</f>
-        <v/>
       </c>
     </row>
     <row r="11">
@@ -3422,20 +3402,20 @@
           <t>Bill Pay:Orange &amp; Rockland 879293 5Bq1P6Kr</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
-      <c r="N11" s="3" t="n"/>
-      <c r="O11" s="3">
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2">
         <f>SUM(B11,C11,D11,E11,F11,G11,H11,I11,J11,K11,L11,M11,N11,Q11)</f>
         <v/>
       </c>
@@ -3451,26 +3431,20 @@
           <t>Bill Pay:Veolia Water New Y 200045 6Bu1T6Kr</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3">
-        <f>300.00</f>
-        <v/>
-      </c>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
-      <c r="M12" s="3" t="n"/>
-      <c r="N12" s="3">
-        <f>300.00</f>
-        <v/>
-      </c>
-      <c r="O12" s="3">
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2">
         <f>SUM(B12,C12,D12,E12,F12,G12,H12,I12,J12,K12,L12,M12,N12,Q12)</f>
         <v/>
       </c>
@@ -3478,10 +3452,6 @@
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
-      </c>
-      <c r="Q12" s="5">
-        <f>300.00</f>
-        <v/>
       </c>
     </row>
     <row r="13">
@@ -3490,20 +3460,20 @@
           <t>Bill Pay:Veolia Water New Y 200054 Hbu1T6Kr</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3">
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2">
         <f>SUM(B13,C13,D13,E13,F13,G13,H13,I13,J13,K13,L13,M13,N13,Q13)</f>
         <v/>
       </c>
@@ -3519,26 +3489,20 @@
           <t>Citi Card Onlinepayment</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3">
-        <f>975.00</f>
-        <v/>
-      </c>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3">
-        <f>975.00</f>
-        <v/>
-      </c>
-      <c r="O14" s="3">
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2">
         <f>SUM(B14,C14,D14,E14,F14,G14,H14,I14,J14,K14,L14,M14,N14,Q14)</f>
         <v/>
       </c>
@@ -3546,10 +3510,6 @@
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
-      </c>
-      <c r="Q14" s="5">
-        <f>975.00</f>
-        <v/>
       </c>
     </row>
     <row r="15">
@@ -3558,26 +3518,20 @@
           <t>Credit One Bank Payment</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3">
-        <f>817.29</f>
-        <v/>
-      </c>
-      <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3">
-        <f>817.29</f>
-        <v/>
-      </c>
-      <c r="O15" s="3">
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n"/>
+      <c r="M15" s="2" t="n"/>
+      <c r="N15" s="2" t="n"/>
+      <c r="O15" s="2">
         <f>SUM(B15,C15,D15,E15,F15,G15,H15,I15,J15,K15,L15,M15,N15,Q15)</f>
         <v/>
       </c>
@@ -3585,10 +3539,6 @@
         <is>
           <t>OFFICE EXPENSE</t>
         </is>
-      </c>
-      <c r="Q15" s="5">
-        <f>817.29</f>
-        <v/>
       </c>
     </row>
     <row r="16">
@@ -3597,20 +3547,20 @@
           <t>Discover Bank Net/Mobile</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="3" t="n"/>
-      <c r="L16" s="3" t="n"/>
-      <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3">
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n"/>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" s="2">
         <f>SUM(B16,C16,D16,E16,F16,G16,H16,I16,J16,K16,L16,M16,N16,Q16)</f>
         <v/>
       </c>
@@ -3626,20 +3576,20 @@
           <t>FIVE GUYS 1522 QSR 000001522 TULSA OK</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
-      <c r="L17" s="3" t="n"/>
-      <c r="M17" s="3" t="n"/>
-      <c r="N17" s="3" t="n"/>
-      <c r="O17" s="3">
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="2" t="n"/>
+      <c r="O17" s="2">
         <f>SUM(B17,C17,D17,E17,F17,G17,H17,I17,J17,K17,L17,M17,N17,Q17)</f>
         <v/>
       </c>
@@ -3655,20 +3605,20 @@
           <t>Huntington Banksil Payment</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
-      <c r="L18" s="3" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3" t="n"/>
-      <c r="O18" s="3">
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n"/>
+      <c r="M18" s="2" t="n"/>
+      <c r="N18" s="2" t="n"/>
+      <c r="O18" s="2">
         <f>SUM(B18,C18,D18,E18,F18,G18,H18,I18,J18,K18,L18,M18,N18,Q18)</f>
         <v/>
       </c>
@@ -3684,26 +3634,20 @@
           <t>Internet Trf To Client-Added Transfer Account</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3">
-        <f>385.77+740.00</f>
-        <v/>
-      </c>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="n"/>
-      <c r="M19" s="3" t="n"/>
-      <c r="N19" s="3">
-        <f>385.77+740.00</f>
-        <v/>
-      </c>
-      <c r="O19" s="3">
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="2" t="n"/>
+      <c r="O19" s="2">
         <f>SUM(B19,C19,D19,E19,F19,G19,H19,I19,J19,K19,L19,M19,N19,Q19)</f>
         <v/>
       </c>
@@ -3711,10 +3655,6 @@
         <is>
           <t>MEALS</t>
         </is>
-      </c>
-      <c r="Q19" s="5">
-        <f>385.77+740.00</f>
-        <v/>
       </c>
     </row>
     <row r="20">
@@ -3723,26 +3663,20 @@
           <t>Irs Usataxpymt</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3">
-        <f>800.00+800.00</f>
-        <v/>
-      </c>
-      <c r="I20" s="3" t="n"/>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="3" t="n"/>
-      <c r="L20" s="3" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="N20" s="3">
-        <f>800.00+800.00</f>
-        <v/>
-      </c>
-      <c r="O20" s="3">
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="2" t="n"/>
+      <c r="O20" s="2">
         <f>SUM(B20,C20,D20,E20,F20,G20,H20,I20,J20,K20,L20,M20,N20,Q20)</f>
         <v/>
       </c>
@@ -3750,10 +3684,6 @@
         <is>
           <t>MEALS</t>
         </is>
-      </c>
-      <c r="Q20" s="5">
-        <f>800.00+800.00</f>
-        <v/>
       </c>
     </row>
     <row r="21">
@@ -3762,26 +3692,20 @@
           <t>Kindercare Portland OR</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3">
-        <f>490.00+120.00</f>
-        <v/>
-      </c>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
-      <c r="M21" s="3" t="n"/>
-      <c r="N21" s="3">
-        <f>490.00+120.00</f>
-        <v/>
-      </c>
-      <c r="O21" s="3">
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="n"/>
+      <c r="M21" s="2" t="n"/>
+      <c r="N21" s="2" t="n"/>
+      <c r="O21" s="2">
         <f>SUM(B21,C21,D21,E21,F21,G21,H21,I21,J21,K21,L21,M21,N21,Q21)</f>
         <v/>
       </c>
@@ -3789,10 +3713,6 @@
         <is>
           <t>MEALS</t>
         </is>
-      </c>
-      <c r="Q21" s="5">
-        <f>490.00+120.00</f>
-        <v/>
       </c>
     </row>
     <row r="22">
@@ -3801,26 +3721,20 @@
           <t>No1 Sushi 88 Corkbbo ACH</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3">
-        <f>4000.00</f>
-        <v/>
-      </c>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3">
-        <f>4000.00</f>
-        <v/>
-      </c>
-      <c r="O22" s="3">
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="2" t="n"/>
+      <c r="O22" s="2">
         <f>SUM(B22,C22,D22,E22,F22,G22,H22,I22,J22,K22,L22,M22,N22,Q22)</f>
         <v/>
       </c>
@@ -3828,10 +3742,6 @@
         <is>
           <t>MEALS</t>
         </is>
-      </c>
-      <c r="Q22" s="5">
-        <f>4000.00</f>
-        <v/>
       </c>
     </row>
     <row r="23">
@@ -3840,20 +3750,20 @@
           <t>NORDSTROM DIRECT http://shop.nordstrom WA</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3" t="n"/>
-      <c r="O23" s="3">
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="n"/>
+      <c r="N23" s="2" t="n"/>
+      <c r="O23" s="2">
         <f>SUM(B23,C23,D23,E23,F23,G23,H23,I23,J23,K23,L23,M23,N23,Q23)</f>
         <v/>
       </c>
@@ -3869,26 +3779,20 @@
           <t>Nys Dtf Pit Tax Paymnt</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3">
-        <f>200.00+200.00</f>
-        <v/>
-      </c>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3">
-        <f>200.00+200.00</f>
-        <v/>
-      </c>
-      <c r="O24" s="3">
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
+      <c r="M24" s="2" t="n"/>
+      <c r="N24" s="2" t="n"/>
+      <c r="O24" s="2">
         <f>SUM(B24,C24,D24,E24,F24,G24,H24,I24,J24,K24,L24,M24,N24,Q24)</f>
         <v/>
       </c>
@@ -3896,10 +3800,6 @@
         <is>
           <t>MEALS</t>
         </is>
-      </c>
-      <c r="Q24" s="5">
-        <f>200.00+200.00</f>
-        <v/>
       </c>
     </row>
     <row r="25">
@@ -3908,20 +3808,20 @@
           <t>PANDA EXPRESS TACOMA WA</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
-      <c r="L25" s="3" t="n"/>
-      <c r="M25" s="3" t="n"/>
-      <c r="N25" s="3" t="n"/>
-      <c r="O25" s="3">
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
+      <c r="M25" s="2" t="n"/>
+      <c r="N25" s="2" t="n"/>
+      <c r="O25" s="2">
         <f>SUM(B25,C25,D25,E25,F25,G25,H25,I25,J25,K25,L25,M25,N25,Q25)</f>
         <v/>
       </c>
@@ -3937,20 +3837,20 @@
           <t>Paypal Inst Xfer</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="n"/>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
-      <c r="O26" s="3">
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="n"/>
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2" t="n"/>
+      <c r="O26" s="2">
         <f>SUM(B26,C26,D26,E26,F26,G26,H26,I26,J26,K26,L26,M26,N26,Q26)</f>
         <v/>
       </c>
@@ -3966,26 +3866,20 @@
           <t>POS Mac Amazon.Com*9O5 Seattle WA</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3">
-        <f>26.57</f>
-        <v/>
-      </c>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="3" t="n"/>
-      <c r="L27" s="3" t="n"/>
-      <c r="M27" s="3" t="n"/>
-      <c r="N27" s="3">
-        <f>26.57</f>
-        <v/>
-      </c>
-      <c r="O27" s="3">
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="n"/>
+      <c r="K27" s="2" t="n"/>
+      <c r="L27" s="2" t="n"/>
+      <c r="M27" s="2" t="n"/>
+      <c r="N27" s="2" t="n"/>
+      <c r="O27" s="2">
         <f>SUM(B27,C27,D27,E27,F27,G27,H27,I27,J27,K27,L27,M27,N27,Q27)</f>
         <v/>
       </c>
@@ -3993,10 +3887,6 @@
         <is>
           <t>MEALS</t>
         </is>
-      </c>
-      <c r="Q27" s="5">
-        <f>26.57</f>
-        <v/>
       </c>
     </row>
     <row r="28">
@@ -4005,20 +3895,20 @@
           <t>POS Mac Amazon.Com*Au5 Seattle WA</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="n"/>
-      <c r="K28" s="3" t="n"/>
-      <c r="L28" s="3" t="n"/>
-      <c r="M28" s="3" t="n"/>
-      <c r="N28" s="3" t="n"/>
-      <c r="O28" s="3">
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="n"/>
+      <c r="K28" s="2" t="n"/>
+      <c r="L28" s="2" t="n"/>
+      <c r="M28" s="2" t="n"/>
+      <c r="N28" s="2" t="n"/>
+      <c r="O28" s="2">
         <f>SUM(B28,C28,D28,E28,F28,G28,H28,I28,J28,K28,L28,M28,N28,Q28)</f>
         <v/>
       </c>
@@ -4034,20 +3924,20 @@
           <t>POS Mac Amazon.Com*Bq9 Seattle WA</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="3" t="n"/>
-      <c r="K29" s="3" t="n"/>
-      <c r="L29" s="3" t="n"/>
-      <c r="M29" s="3" t="n"/>
-      <c r="N29" s="3" t="n"/>
-      <c r="O29" s="3">
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="n"/>
+      <c r="K29" s="2" t="n"/>
+      <c r="L29" s="2" t="n"/>
+      <c r="M29" s="2" t="n"/>
+      <c r="N29" s="2" t="n"/>
+      <c r="O29" s="2">
         <f>SUM(B29,C29,D29,E29,F29,G29,H29,I29,J29,K29,L29,M29,N29,Q29)</f>
         <v/>
       </c>
@@ -4063,20 +3953,20 @@
           <t>POS Mac Amazon.Com*Ge2 Seattle WA</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="3" t="n"/>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="3" t="n"/>
-      <c r="K30" s="3" t="n"/>
-      <c r="L30" s="3" t="n"/>
-      <c r="M30" s="3" t="n"/>
-      <c r="N30" s="3" t="n"/>
-      <c r="O30" s="3">
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="n"/>
+      <c r="M30" s="2" t="n"/>
+      <c r="N30" s="2" t="n"/>
+      <c r="O30" s="2">
         <f>SUM(B30,C30,D30,E30,F30,G30,H30,I30,J30,K30,L30,M30,N30,Q30)</f>
         <v/>
       </c>
@@ -4092,20 +3982,20 @@
           <t>POS Mac Amazon.Com*Mz5 Seattle WA</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
-      <c r="F31" s="3" t="n"/>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="3" t="n"/>
-      <c r="I31" s="3" t="n"/>
-      <c r="J31" s="3" t="n"/>
-      <c r="K31" s="3" t="n"/>
-      <c r="L31" s="3" t="n"/>
-      <c r="M31" s="3" t="n"/>
-      <c r="N31" s="3" t="n"/>
-      <c r="O31" s="3">
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="n"/>
+      <c r="M31" s="2" t="n"/>
+      <c r="N31" s="2" t="n"/>
+      <c r="O31" s="2">
         <f>SUM(B31,C31,D31,E31,F31,G31,H31,I31,J31,K31,L31,M31,N31,Q31)</f>
         <v/>
       </c>
@@ -4121,26 +4011,20 @@
           <t>POS Mac Amazon.Com*Nx6 Seattle WA</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n"/>
-      <c r="C32" s="3" t="n"/>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="3" t="n"/>
-      <c r="F32" s="3" t="n"/>
-      <c r="G32" s="3" t="n"/>
-      <c r="H32" s="3">
-        <f>75.40</f>
-        <v/>
-      </c>
-      <c r="I32" s="3" t="n"/>
-      <c r="J32" s="3" t="n"/>
-      <c r="K32" s="3" t="n"/>
-      <c r="L32" s="3" t="n"/>
-      <c r="M32" s="3" t="n"/>
-      <c r="N32" s="3">
-        <f>75.40</f>
-        <v/>
-      </c>
-      <c r="O32" s="3">
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n"/>
+      <c r="M32" s="2" t="n"/>
+      <c r="N32" s="2" t="n"/>
+      <c r="O32" s="2">
         <f>SUM(B32,C32,D32,E32,F32,G32,H32,I32,J32,K32,L32,M32,N32,Q32)</f>
         <v/>
       </c>
@@ -4148,10 +4032,6 @@
         <is>
           <t>SUPPLY</t>
         </is>
-      </c>
-      <c r="Q32" s="5">
-        <f>75.40</f>
-        <v/>
       </c>
     </row>
     <row r="33">
@@ -4160,26 +4040,20 @@
           <t>POS Mac Amazon.Com*Sb8 Seattle WA</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n"/>
-      <c r="G33" s="3" t="n"/>
-      <c r="H33" s="3">
-        <f>18.75</f>
-        <v/>
-      </c>
-      <c r="I33" s="3" t="n"/>
-      <c r="J33" s="3" t="n"/>
-      <c r="K33" s="3" t="n"/>
-      <c r="L33" s="3" t="n"/>
-      <c r="M33" s="3" t="n"/>
-      <c r="N33" s="3">
-        <f>18.75</f>
-        <v/>
-      </c>
-      <c r="O33" s="3">
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="n"/>
+      <c r="M33" s="2" t="n"/>
+      <c r="N33" s="2" t="n"/>
+      <c r="O33" s="2">
         <f>SUM(B33,C33,D33,E33,F33,G33,H33,I33,J33,K33,L33,M33,N33,Q33)</f>
         <v/>
       </c>
@@ -4187,10 +4061,6 @@
         <is>
           <t>SUPPLY</t>
         </is>
-      </c>
-      <c r="Q33" s="5">
-        <f>18.75</f>
-        <v/>
       </c>
     </row>
     <row r="34">
@@ -4199,20 +4069,20 @@
           <t>POS Mac Amazon.Com*TN0 Seattle WA</t>
         </is>
       </c>
-      <c r="B34" s="3" t="n"/>
-      <c r="C34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34" s="3" t="n"/>
-      <c r="G34" s="3" t="n"/>
-      <c r="H34" s="3" t="n"/>
-      <c r="I34" s="3" t="n"/>
-      <c r="J34" s="3" t="n"/>
-      <c r="K34" s="3" t="n"/>
-      <c r="L34" s="3" t="n"/>
-      <c r="M34" s="3" t="n"/>
-      <c r="N34" s="3" t="n"/>
-      <c r="O34" s="3">
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="2" t="n"/>
+      <c r="L34" s="2" t="n"/>
+      <c r="M34" s="2" t="n"/>
+      <c r="N34" s="2" t="n"/>
+      <c r="O34" s="2">
         <f>SUM(B34,C34,D34,E34,F34,G34,H34,I34,J34,K34,L34,M34,N34,Q34)</f>
         <v/>
       </c>
@@ -4228,20 +4098,20 @@
           <t>POS Mac Amazon.Com*V25 Seattle WA</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n"/>
-      <c r="J35" s="3" t="n"/>
-      <c r="K35" s="3" t="n"/>
-      <c r="L35" s="3" t="n"/>
-      <c r="M35" s="3" t="n"/>
-      <c r="N35" s="3" t="n"/>
-      <c r="O35" s="3">
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="n"/>
+      <c r="M35" s="2" t="n"/>
+      <c r="N35" s="2" t="n"/>
+      <c r="O35" s="2">
         <f>SUM(B35,C35,D35,E35,F35,G35,H35,I35,J35,K35,L35,M35,N35,Q35)</f>
         <v/>
       </c>
@@ -4257,20 +4127,20 @@
           <t>POS Mac Amazon.Com*Yr6 Seattle WA</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="n"/>
-      <c r="G36" s="3" t="n"/>
-      <c r="H36" s="3" t="n"/>
-      <c r="I36" s="3" t="n"/>
-      <c r="J36" s="3" t="n"/>
-      <c r="K36" s="3" t="n"/>
-      <c r="L36" s="3" t="n"/>
-      <c r="M36" s="3" t="n"/>
-      <c r="N36" s="3" t="n"/>
-      <c r="O36" s="3">
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="n"/>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="n"/>
+      <c r="M36" s="2" t="n"/>
+      <c r="N36" s="2" t="n"/>
+      <c r="O36" s="2">
         <f>SUM(B36,C36,D36,E36,F36,G36,H36,I36,J36,K36,L36,M36,N36,Q36)</f>
         <v/>
       </c>
@@ -4286,20 +4156,20 @@
           <t>POS Mac Amazon.Com*Za2 Seattle WA</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n"/>
-      <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
-      <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
-      <c r="H37" s="3" t="n"/>
-      <c r="I37" s="3" t="n"/>
-      <c r="J37" s="3" t="n"/>
-      <c r="K37" s="3" t="n"/>
-      <c r="L37" s="3" t="n"/>
-      <c r="M37" s="3" t="n"/>
-      <c r="N37" s="3" t="n"/>
-      <c r="O37" s="3">
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
+      <c r="M37" s="2" t="n"/>
+      <c r="N37" s="2" t="n"/>
+      <c r="O37" s="2">
         <f>SUM(B37,C37,D37,E37,F37,G37,H37,I37,J37,K37,L37,M37,N37,Q37)</f>
         <v/>
       </c>
@@ -4315,26 +4185,20 @@
           <t>Prog Casualty Ins Prem</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n"/>
-      <c r="C38" s="3" t="n"/>
-      <c r="D38" s="3" t="n"/>
-      <c r="E38" s="3" t="n"/>
-      <c r="F38" s="3" t="n"/>
-      <c r="G38" s="3" t="n"/>
-      <c r="H38" s="3">
-        <f>930.52</f>
-        <v/>
-      </c>
-      <c r="I38" s="3" t="n"/>
-      <c r="J38" s="3" t="n"/>
-      <c r="K38" s="3" t="n"/>
-      <c r="L38" s="3" t="n"/>
-      <c r="M38" s="3" t="n"/>
-      <c r="N38" s="3">
-        <f>930.52</f>
-        <v/>
-      </c>
-      <c r="O38" s="3">
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="n"/>
+      <c r="J38" s="2" t="n"/>
+      <c r="K38" s="2" t="n"/>
+      <c r="L38" s="2" t="n"/>
+      <c r="M38" s="2" t="n"/>
+      <c r="N38" s="2" t="n"/>
+      <c r="O38" s="2">
         <f>SUM(B38,C38,D38,E38,F38,G38,H38,I38,J38,K38,L38,M38,N38,Q38)</f>
         <v/>
       </c>
@@ -4342,10 +4206,6 @@
         <is>
           <t>SUPPLY</t>
         </is>
-      </c>
-      <c r="Q38" s="5">
-        <f>930.52</f>
-        <v/>
       </c>
     </row>
     <row r="39">
@@ -4354,20 +4214,20 @@
           <t>WHOLEFDS CHB #10588 000010588 UNIVERSITY PL WA</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n"/>
-      <c r="C39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
-      <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
-      <c r="J39" s="3" t="n"/>
-      <c r="K39" s="3" t="n"/>
-      <c r="L39" s="3" t="n"/>
-      <c r="M39" s="3" t="n"/>
-      <c r="N39" s="3" t="n"/>
-      <c r="O39" s="3">
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
+      <c r="J39" s="2" t="n"/>
+      <c r="K39" s="2" t="n"/>
+      <c r="L39" s="2" t="n"/>
+      <c r="M39" s="2" t="n"/>
+      <c r="N39" s="2" t="n"/>
+      <c r="O39" s="2">
         <f>SUM(B39,C39,D39,E39,F39,G39,H39,I39,J39,K39,L39,M39,N39,Q39)</f>
         <v/>
       </c>
@@ -4383,26 +4243,20 @@
           <t>Withdrawal Branch 0964 New York</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="n"/>
-      <c r="H40" s="3">
-        <f>1000.00+3200.00</f>
-        <v/>
-      </c>
-      <c r="I40" s="3" t="n"/>
-      <c r="J40" s="3" t="n"/>
-      <c r="K40" s="3" t="n"/>
-      <c r="L40" s="3" t="n"/>
-      <c r="M40" s="3" t="n"/>
-      <c r="N40" s="3">
-        <f>1000.00+3200.00</f>
-        <v/>
-      </c>
-      <c r="O40" s="3">
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
+      <c r="K40" s="2" t="n"/>
+      <c r="L40" s="2" t="n"/>
+      <c r="M40" s="2" t="n"/>
+      <c r="N40" s="2" t="n"/>
+      <c r="O40" s="2">
         <f>SUM(B40,C40,D40,E40,F40,G40,H40,I40,J40,K40,L40,M40,N40,Q40)</f>
         <v/>
       </c>
@@ -4410,10 +4264,6 @@
         <is>
           <t>SUPPLY</t>
         </is>
-      </c>
-      <c r="Q40" s="5">
-        <f>1000.00+3200.00</f>
-        <v/>
       </c>
     </row>
     <row r="41">
@@ -4422,64 +4272,64 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B41" s="3">
+      <c r="B41" s="2">
         <f>SUM(B2:B40)</f>
         <v/>
       </c>
-      <c r="C41" s="3">
+      <c r="C41" s="2">
         <f>SUM(C2:C40)</f>
         <v/>
       </c>
-      <c r="D41" s="3">
+      <c r="D41" s="2">
         <f>SUM(D2:D40)</f>
         <v/>
       </c>
-      <c r="E41" s="3">
+      <c r="E41" s="2">
         <f>SUM(E2:E40)</f>
         <v/>
       </c>
-      <c r="F41" s="3">
+      <c r="F41" s="2">
         <f>SUM(F2:F40)</f>
         <v/>
       </c>
-      <c r="G41" s="3">
+      <c r="G41" s="2">
         <f>SUM(G2:G40)</f>
         <v/>
       </c>
-      <c r="H41" s="3">
+      <c r="H41" s="2">
         <f>SUM(H2:H40)</f>
         <v/>
       </c>
-      <c r="I41" s="3">
+      <c r="I41" s="2">
         <f>SUM(I2:I40)</f>
         <v/>
       </c>
-      <c r="J41" s="3">
+      <c r="J41" s="2">
         <f>SUM(J2:J40)</f>
         <v/>
       </c>
-      <c r="K41" s="3">
+      <c r="K41" s="2">
         <f>SUM(K2:K40)</f>
         <v/>
       </c>
-      <c r="L41" s="3">
+      <c r="L41" s="2">
         <f>SUM(L2:L40)</f>
         <v/>
       </c>
-      <c r="M41" s="3">
+      <c r="M41" s="2">
         <f>SUM(M2:M40)</f>
         <v/>
       </c>
-      <c r="N41" s="3">
+      <c r="N41" s="2">
         <f>SUM(N2:N40)</f>
         <v/>
       </c>
-      <c r="O41" s="3">
+      <c r="O41" s="2">
         <f>SUM(B41,C41,D41,E41,F41,G41,H41,I41,J41,K41,L41,M41,N41,Q41)</f>
         <v/>
       </c>
       <c r="P41" s="1" t="n"/>
-      <c r="Q41" s="5">
+      <c r="Q41" s="4">
         <f>SUM(Q2:Q40)</f>
         <v/>
       </c>
@@ -4497,7 +4347,9 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1"/>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>